<commit_message>
Better 8-bit `shuffle` using XOR tree
- Improves `shuffleVar_u8` performance by replacing scalar array load with XOR tree method. (0-100% faster, save size)
- Updated excel files to reflect these changes
</commit_message>
<xml_diff>
--- a/external/InstructionCost.xlsx
+++ b/external/InstructionCost.xlsx
@@ -1,23 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\walte\Desktop\Coding\Filling SIMD gaps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC0983AC-4685-4CB9-999E-FB31977DE637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F29AFA-CAE3-4C54-98C6-4FE8C40F5DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{0228E47D-794C-431C-A2A8-62B0A8D25E03}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{0228E47D-794C-431C-A2A8-62B0A8D25E03}"/>
   </bookViews>
   <sheets>
     <sheet name="Emulated" sheetId="1" r:id="rId1"/>
-    <sheet name="SSE operations" sheetId="2" r:id="rId2"/>
-    <sheet name="enums" sheetId="3" r:id="rId3"/>
+    <sheet name="Extention operation support" sheetId="2" r:id="rId2"/>
+    <sheet name="MMX timeline" sheetId="4" r:id="rId3"/>
+    <sheet name="enums" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Extention operation support'!$A$38:$K$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MMX timeline'!$A$1:$I$24</definedName>
+  </definedNames>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -371,7 +376,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="180">
   <si>
     <t>s8</t>
   </si>
@@ -905,6 +910,12 @@
   </si>
   <si>
     <t>madd[ubs]</t>
+  </si>
+  <si>
+    <t>enums</t>
+  </si>
+  <si>
+    <t>MMX</t>
   </si>
 </sst>
 </file>
@@ -1015,7 +1026,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -1217,11 +1228,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1352,6 +1400,9 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1419,75 +1470,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="23">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
+          <bgColor rgb="FFFFFF89"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1570,10 +1557,107 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF9DE7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFBCFF79"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB9FF2D"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00DE00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF008E00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFFF89"/>
       <color rgb="FF920000"/>
       <color rgb="FF00DE00"/>
       <color rgb="FF008E00"/>
@@ -1583,7 +1667,6 @@
       <color rgb="FFCCFF66"/>
       <color rgb="FFA1FF43"/>
       <color rgb="FFBCFF79"/>
-      <color rgb="FF99FF33"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1915,12 +1998,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D60BA8C6-A487-451B-A2BD-8E39E20BCE51}">
   <dimension ref="A1:N43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.5703125" customWidth="1"/>
+    <col min="1" max="1" width="34.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="24" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="24" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
@@ -1952,7 +2035,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>151</v>
       </c>
@@ -1967,7 +2050,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
@@ -2002,7 +2085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
@@ -2037,7 +2120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
@@ -2072,7 +2155,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>13</v>
       </c>
@@ -2107,7 +2190,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>14</v>
       </c>
@@ -2126,7 +2209,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>35</v>
       </c>
@@ -2161,7 +2244,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>34</v>
       </c>
@@ -2196,7 +2279,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>33</v>
       </c>
@@ -2231,26 +2314,26 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="51">
         <v>25</v>
       </c>
-      <c r="C11" s="49"/>
-      <c r="D11" s="49">
+      <c r="C11" s="52"/>
+      <c r="D11" s="52">
         <v>13</v>
       </c>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49">
+      <c r="E11" s="52"/>
+      <c r="F11" s="52">
         <v>12</v>
       </c>
-      <c r="G11" s="49"/>
-      <c r="H11" s="49">
+      <c r="G11" s="52"/>
+      <c r="H11" s="52">
         <v>6</v>
       </c>
-      <c r="I11" s="50"/>
+      <c r="I11" s="53"/>
       <c r="J11" s="1" t="s">
         <v>36</v>
       </c>
@@ -2258,26 +2341,26 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B12" s="48">
+      <c r="B12" s="51">
         <v>27</v>
       </c>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49">
+      <c r="C12" s="52"/>
+      <c r="D12" s="52">
         <v>21</v>
       </c>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49">
+      <c r="E12" s="52"/>
+      <c r="F12" s="52">
         <v>19</v>
       </c>
-      <c r="G12" s="49"/>
-      <c r="H12" s="49">
+      <c r="G12" s="52"/>
+      <c r="H12" s="52">
         <v>6</v>
       </c>
-      <c r="I12" s="50"/>
+      <c r="I12" s="53"/>
       <c r="J12" s="1" t="s">
         <v>36</v>
       </c>
@@ -2285,26 +2368,26 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="48">
-        <v>85</v>
-      </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49">
+      <c r="B13" s="51">
+        <v>86</v>
+      </c>
+      <c r="C13" s="52"/>
+      <c r="D13" s="52">
         <v>19</v>
       </c>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49">
+      <c r="E13" s="52"/>
+      <c r="F13" s="52">
         <v>16</v>
       </c>
-      <c r="G13" s="49"/>
-      <c r="H13" s="49">
+      <c r="G13" s="52"/>
+      <c r="H13" s="52">
         <v>9</v>
       </c>
-      <c r="I13" s="50"/>
+      <c r="I13" s="53"/>
       <c r="J13" s="1" t="s">
         <v>36</v>
       </c>
@@ -2312,7 +2395,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>15</v>
       </c>
@@ -2335,7 +2418,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>16</v>
       </c>
@@ -2366,7 +2449,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>37</v>
       </c>
@@ -2397,7 +2480,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>17</v>
       </c>
@@ -2420,7 +2503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>18</v>
       </c>
@@ -2447,26 +2530,26 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="48">
+      <c r="B19" s="51">
         <v>7</v>
       </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49">
-        <v>1</v>
-      </c>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49">
+      <c r="C19" s="52"/>
+      <c r="D19" s="52">
+        <v>1</v>
+      </c>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52">
         <v>8</v>
       </c>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49">
+      <c r="G19" s="52"/>
+      <c r="H19" s="52">
         <v>13</v>
       </c>
-      <c r="I19" s="50"/>
+      <c r="I19" s="53"/>
       <c r="J19" s="1" t="s">
         <v>36</v>
       </c>
@@ -2474,7 +2557,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>20</v>
       </c>
@@ -2509,7 +2592,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>21</v>
       </c>
@@ -2544,7 +2627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>71</v>
       </c>
@@ -2579,7 +2662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>144</v>
       </c>
@@ -2613,13 +2696,13 @@
       <c r="K23" s="6">
         <v>1</v>
       </c>
-      <c r="L23" s="46" t="s">
+      <c r="L23" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="M23" s="47"/>
-      <c r="N23" s="47"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="M23" s="50"/>
+      <c r="N23" s="50"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>147</v>
       </c>
@@ -2641,11 +2724,11 @@
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="6"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="47"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L24" s="49"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="50"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>145</v>
       </c>
@@ -2671,11 +2754,11 @@
       <c r="K25" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="L25" s="46"/>
-      <c r="M25" s="47"/>
-      <c r="N25" s="47"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L25" s="49"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>148</v>
       </c>
@@ -2697,11 +2780,11 @@
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="47"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L26" s="49"/>
+      <c r="M26" s="50"/>
+      <c r="N26" s="50"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
         <v>36</v>
       </c>
@@ -2733,7 +2816,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>22</v>
       </c>
@@ -2768,26 +2851,26 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B29" s="48">
-        <v>1</v>
-      </c>
-      <c r="C29" s="49"/>
-      <c r="D29" s="49">
-        <v>1</v>
-      </c>
-      <c r="E29" s="49"/>
-      <c r="F29" s="49">
-        <v>1</v>
-      </c>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49">
+      <c r="B29" s="51">
+        <v>1</v>
+      </c>
+      <c r="C29" s="52"/>
+      <c r="D29" s="52">
+        <v>1</v>
+      </c>
+      <c r="E29" s="52"/>
+      <c r="F29" s="52">
+        <v>1</v>
+      </c>
+      <c r="G29" s="52"/>
+      <c r="H29" s="52">
         <v>3</v>
       </c>
-      <c r="I29" s="50"/>
+      <c r="I29" s="53"/>
       <c r="J29" s="1">
         <v>1</v>
       </c>
@@ -2795,7 +2878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>25</v>
       </c>
@@ -2830,7 +2913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>26</v>
       </c>
@@ -2865,7 +2948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>27</v>
       </c>
@@ -2894,7 +2977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>28</v>
       </c>
@@ -2923,7 +3006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B34" s="5" t="s">
         <v>36</v>
       </c>
@@ -2955,7 +3038,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>29</v>
       </c>
@@ -2990,7 +3073,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>30</v>
       </c>
@@ -3025,7 +3108,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
         <v>31</v>
       </c>
@@ -3060,7 +3143,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
         <v>32</v>
       </c>
@@ -3095,7 +3178,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>38</v>
       </c>
@@ -3124,7 +3207,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>75</v>
       </c>
@@ -3159,7 +3242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>76</v>
       </c>
@@ -3194,7 +3277,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>149</v>
       </c>
@@ -3229,7 +3312,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>150</v>
       </c>
@@ -3288,6 +3371,11 @@
     <mergeCell ref="F29:G29"/>
     <mergeCell ref="H29:I29"/>
   </mergeCells>
+  <conditionalFormatting sqref="B11:C11 B12:K12 B13 D13 B14:K26 B3:K10 F11:K11 F13 H13 J13:K13 B29:K33 B36:K43">
+    <cfRule type="containsBlanks" dxfId="22" priority="12">
+      <formula>LEN(TRIM(B3))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11 I22 C22 B23:C24 E23:E24 G22:G24 B12:B13 D12:D13">
     <cfRule type="colorScale" priority="10">
       <colorScale>
@@ -3311,13 +3399,8 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:K10 F11:F13 H11:H13 J11:K13 B14:K18 B19 D19 F19 H19 J19:K19 B20:K28 B29 D29 F29 H29 J29:K29 B30:K43">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="1" operator="equal">
       <formula>"#"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:K10 B13 D13 B14:K26 F13 H13 J13:K13 B29:K33 B36:K43 B12:K12 B11:C11 F11:K11">
-    <cfRule type="containsBlanks" dxfId="3" priority="12">
-      <formula>LEN(TRIM(B3))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3329,16 +3412,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EB52227-ACC2-4A13-BAC7-C7465281EE66}">
   <dimension ref="A1:N76"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.28515625" customWidth="1"/>
-    <col min="2" max="11" width="9.140625" style="1"/>
-    <col min="12" max="12" width="2.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" style="19" customWidth="1"/>
-    <col min="14" max="14" width="68.7109375" style="20" customWidth="1"/>
+    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="2" max="11" width="9.109375" style="1"/>
+    <col min="12" max="12" width="2.5546875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" style="19" customWidth="1"/>
+    <col min="14" max="14" width="68.6640625" style="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="17" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>23</v>
       </c>
@@ -3374,26 +3457,26 @@
       </c>
       <c r="L1" s="16"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I2" s="65"/>
+      <c r="B2" s="66" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="I2" s="68"/>
       <c r="J2" s="31" t="s">
         <v>83</v>
       </c>
@@ -3405,26 +3488,26 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="I3" s="59"/>
+      <c r="B3" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" s="62"/>
       <c r="J3" s="27" t="s">
         <v>83</v>
       </c>
@@ -3436,7 +3519,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -3467,7 +3550,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
@@ -3498,24 +3581,24 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34"/>
-      <c r="D6" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53" t="s">
+      <c r="D6" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53" t="s">
+      <c r="G6" s="56"/>
+      <c r="H6" s="56" t="s">
         <v>167</v>
       </c>
-      <c r="I6" s="54"/>
+      <c r="I6" s="57"/>
       <c r="J6" s="33" t="s">
         <v>84</v>
       </c>
@@ -3527,7 +3610,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>65</v>
       </c>
@@ -3554,7 +3637,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>66</v>
       </c>
@@ -3581,7 +3664,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>60</v>
       </c>
@@ -3604,7 +3687,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>14</v>
       </c>
@@ -3627,7 +3710,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>15</v>
       </c>
@@ -3662,7 +3745,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>39</v>
       </c>
@@ -3685,7 +3768,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>46</v>
       </c>
@@ -3724,7 +3807,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>47</v>
       </c>
@@ -3763,7 +3846,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>18</v>
       </c>
@@ -3802,7 +3885,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>17</v>
       </c>
@@ -3841,22 +3924,22 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53" t="s">
+      <c r="B17" s="55"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="53"/>
-      <c r="F17" s="53" t="s">
+      <c r="E17" s="56"/>
+      <c r="F17" s="56" t="s">
         <v>80</v>
       </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="54"/>
+      <c r="G17" s="56"/>
+      <c r="H17" s="56"/>
+      <c r="I17" s="57"/>
       <c r="J17" s="33" t="s">
         <v>79</v>
       </c>
@@ -3868,22 +3951,22 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="51"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="58" t="s">
+      <c r="B18" s="54"/>
+      <c r="C18" s="61"/>
+      <c r="D18" s="61" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="58"/>
-      <c r="F18" s="58" t="s">
+      <c r="E18" s="61"/>
+      <c r="F18" s="61" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="58"/>
-      <c r="H18" s="58"/>
-      <c r="I18" s="59"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="62"/>
       <c r="J18" s="27" t="s">
         <v>79</v>
       </c>
@@ -3895,7 +3978,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>57</v>
       </c>
@@ -3920,7 +4003,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>59</v>
       </c>
@@ -3945,7 +4028,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>62</v>
       </c>
@@ -3966,7 +4049,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>63</v>
       </c>
@@ -3987,7 +4070,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>67</v>
       </c>
@@ -4008,7 +4091,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>95</v>
       </c>
@@ -4041,7 +4124,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>94</v>
       </c>
@@ -4078,7 +4161,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>69</v>
       </c>
@@ -4117,7 +4200,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>71</v>
       </c>
@@ -4140,7 +4223,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>85</v>
       </c>
@@ -4163,55 +4246,55 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B29" s="52"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="53"/>
-      <c r="G29" s="53"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="52"/>
-      <c r="K29" s="54"/>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B29" s="55"/>
+      <c r="C29" s="56"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="56"/>
+      <c r="H29" s="56"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="55"/>
+      <c r="K29" s="57"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="55"/>
-      <c r="C30" s="56"/>
-      <c r="D30" s="56"/>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="57"/>
-      <c r="J30" s="55"/>
-      <c r="K30" s="57"/>
+      <c r="B30" s="58"/>
+      <c r="C30" s="59"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="59"/>
+      <c r="G30" s="59"/>
+      <c r="H30" s="59"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="60"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53" t="s">
+      <c r="B31" s="55" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="G31" s="56"/>
+      <c r="H31" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="I31" s="54"/>
+      <c r="I31" s="57"/>
       <c r="J31" s="33" t="s">
         <v>83</v>
       </c>
@@ -4223,26 +4306,26 @@
         <v>116</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="51" t="s">
+      <c r="B32" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="58"/>
-      <c r="D32" s="58" t="s">
+      <c r="C32" s="61"/>
+      <c r="D32" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="E32" s="58"/>
-      <c r="F32" s="58" t="s">
+      <c r="E32" s="61"/>
+      <c r="F32" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="G32" s="58"/>
-      <c r="H32" s="58" t="s">
+      <c r="G32" s="61"/>
+      <c r="H32" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="I32" s="59"/>
+      <c r="I32" s="62"/>
       <c r="J32" s="27" t="s">
         <v>83</v>
       </c>
@@ -4251,38 +4334,38 @@
       </c>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="58" t="s">
+      <c r="B33" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="D33" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E33" s="58" t="s">
+      <c r="D33" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E33" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="F33" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="G33" s="58" t="s">
+      <c r="F33" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="G33" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="H33" s="58" t="s">
+      <c r="H33" s="61" t="s">
         <v>82</v>
       </c>
-      <c r="I33" s="59" t="s">
+      <c r="I33" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="J33" s="51" t="s">
+      <c r="J33" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="K33" s="59" t="s">
+      <c r="K33" s="62" t="s">
         <v>78</v>
       </c>
       <c r="L33" s="18"/>
@@ -4290,107 +4373,107 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="51"/>
-      <c r="C34" s="58"/>
-      <c r="D34" s="58"/>
-      <c r="E34" s="58"/>
-      <c r="F34" s="58"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="58"/>
-      <c r="I34" s="59"/>
-      <c r="J34" s="51"/>
-      <c r="K34" s="59"/>
+      <c r="B34" s="54"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="54"/>
+      <c r="K34" s="62"/>
       <c r="L34" s="18"/>
       <c r="M34" s="19" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="51" t="s">
+      <c r="B35" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="C35" s="58" t="s">
+      <c r="C35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="D35" s="58" t="s">
+      <c r="D35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="E35" s="58" t="s">
+      <c r="E35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="F35" s="58" t="s">
+      <c r="F35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="G35" s="58" t="s">
+      <c r="G35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="H35" s="58" t="s">
+      <c r="H35" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="I35" s="59" t="s">
+      <c r="I35" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="J35" s="51" t="s">
+      <c r="J35" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="K35" s="59" t="s">
+      <c r="K35" s="62" t="s">
         <v>78</v>
       </c>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="55"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="57"/>
-      <c r="J36" s="55"/>
-      <c r="K36" s="57"/>
+      <c r="B36" s="58"/>
+      <c r="C36" s="59"/>
+      <c r="D36" s="59"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="59"/>
+      <c r="G36" s="59"/>
+      <c r="H36" s="59"/>
+      <c r="I36" s="60"/>
+      <c r="J36" s="58"/>
+      <c r="K36" s="60"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B37" s="52"/>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="53"/>
-      <c r="G37" s="53"/>
-      <c r="H37" s="53"/>
-      <c r="I37" s="54"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="54"/>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B37" s="55"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="57"/>
+      <c r="J37" s="55"/>
+      <c r="K37" s="57"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="55"/>
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="57"/>
-      <c r="J38" s="55"/>
-      <c r="K38" s="57"/>
+      <c r="B38" s="58"/>
+      <c r="C38" s="59"/>
+      <c r="D38" s="59"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="59"/>
+      <c r="G38" s="59"/>
+      <c r="H38" s="59"/>
+      <c r="I38" s="60"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="60"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>90</v>
       </c>
@@ -4425,11 +4508,11 @@
         <v>84</v>
       </c>
       <c r="L39" s="14"/>
-      <c r="M39" s="66" t="s">
+      <c r="M39" s="69" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>91</v>
       </c>
@@ -4464,9 +4547,9 @@
         <v>84</v>
       </c>
       <c r="L40" s="14"/>
-      <c r="M40" s="66"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M40" s="69"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>92</v>
       </c>
@@ -4501,9 +4584,9 @@
         <v>84</v>
       </c>
       <c r="L41" s="14"/>
-      <c r="M41" s="66"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M41" s="69"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>89</v>
       </c>
@@ -4538,11 +4621,11 @@
         <v>84</v>
       </c>
       <c r="L42" s="14"/>
-      <c r="M42" s="66" t="s">
+      <c r="M42" s="69" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>88</v>
       </c>
@@ -4577,9 +4660,9 @@
         <v>84</v>
       </c>
       <c r="L43" s="14"/>
-      <c r="M43" s="66"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M43" s="69"/>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>87</v>
       </c>
@@ -4614,9 +4697,9 @@
         <v>84</v>
       </c>
       <c r="L44" s="14"/>
-      <c r="M44" s="66"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M44" s="69"/>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>68</v>
       </c>
@@ -4647,7 +4730,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
         <v>75</v>
       </c>
@@ -4678,7 +4761,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>76</v>
       </c>
@@ -4709,7 +4792,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>77</v>
       </c>
@@ -4734,7 +4817,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="43" t="s">
         <v>171</v>
       </c>
@@ -4750,49 +4833,49 @@
       <c r="K49" s="26"/>
       <c r="L49" s="14"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B50" s="51"/>
-      <c r="C50" s="58"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="58"/>
-      <c r="H50" s="58"/>
-      <c r="I50" s="59"/>
-      <c r="J50" s="51"/>
-      <c r="K50" s="59"/>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B50" s="54"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61"/>
+      <c r="F50" s="61"/>
+      <c r="G50" s="61"/>
+      <c r="H50" s="61"/>
+      <c r="I50" s="62"/>
+      <c r="J50" s="54"/>
+      <c r="K50" s="62"/>
       <c r="L50" s="14"/>
     </row>
-    <row r="51" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="55"/>
-      <c r="C51" s="56"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="56"/>
-      <c r="H51" s="56"/>
-      <c r="I51" s="57"/>
-      <c r="J51" s="55"/>
-      <c r="K51" s="57"/>
+      <c r="B51" s="58"/>
+      <c r="C51" s="59"/>
+      <c r="D51" s="59"/>
+      <c r="E51" s="59"/>
+      <c r="F51" s="59"/>
+      <c r="G51" s="59"/>
+      <c r="H51" s="59"/>
+      <c r="I51" s="60"/>
+      <c r="J51" s="58"/>
+      <c r="K51" s="60"/>
       <c r="L51" s="14"/>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B52" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="C52" s="53"/>
-      <c r="D52" s="53"/>
-      <c r="E52" s="53"/>
-      <c r="F52" s="53"/>
-      <c r="G52" s="53"/>
-      <c r="H52" s="53"/>
-      <c r="I52" s="54"/>
+      <c r="B52" s="55" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" s="56"/>
+      <c r="D52" s="56"/>
+      <c r="E52" s="56"/>
+      <c r="F52" s="56"/>
+      <c r="G52" s="56"/>
+      <c r="H52" s="56"/>
+      <c r="I52" s="57"/>
       <c r="J52" s="33" t="s">
         <v>83</v>
       </c>
@@ -4804,20 +4887,20 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B53" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C53" s="58"/>
-      <c r="D53" s="58"/>
-      <c r="E53" s="58"/>
-      <c r="F53" s="58"/>
-      <c r="G53" s="58"/>
-      <c r="H53" s="58"/>
-      <c r="I53" s="59"/>
+      <c r="B53" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C53" s="61"/>
+      <c r="D53" s="61"/>
+      <c r="E53" s="61"/>
+      <c r="F53" s="61"/>
+      <c r="G53" s="61"/>
+      <c r="H53" s="61"/>
+      <c r="I53" s="62"/>
       <c r="J53" s="27" t="s">
         <v>83</v>
       </c>
@@ -4829,20 +4912,20 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B54" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C54" s="58"/>
-      <c r="D54" s="58"/>
-      <c r="E54" s="58"/>
-      <c r="F54" s="58"/>
-      <c r="G54" s="58"/>
-      <c r="H54" s="58"/>
-      <c r="I54" s="59"/>
+      <c r="B54" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C54" s="61"/>
+      <c r="D54" s="61"/>
+      <c r="E54" s="61"/>
+      <c r="F54" s="61"/>
+      <c r="G54" s="61"/>
+      <c r="H54" s="61"/>
+      <c r="I54" s="62"/>
       <c r="J54" s="27" t="s">
         <v>83</v>
       </c>
@@ -4854,20 +4937,20 @@
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B55" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="58"/>
-      <c r="D55" s="58"/>
-      <c r="E55" s="58"/>
-      <c r="F55" s="58"/>
-      <c r="G55" s="58"/>
-      <c r="H55" s="58"/>
-      <c r="I55" s="59"/>
+      <c r="B55" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C55" s="61"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="61"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="61"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="62"/>
       <c r="J55" s="27" t="s">
         <v>83</v>
       </c>
@@ -4879,217 +4962,217 @@
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B56" s="51"/>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="G56" s="58"/>
-      <c r="H56" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="I56" s="59"/>
-      <c r="J56" s="51" t="s">
-        <v>84</v>
-      </c>
-      <c r="K56" s="59"/>
+      <c r="B56" s="54"/>
+      <c r="C56" s="61"/>
+      <c r="D56" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56" s="61"/>
+      <c r="F56" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="G56" s="61"/>
+      <c r="H56" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I56" s="62"/>
+      <c r="J56" s="54" t="s">
+        <v>84</v>
+      </c>
+      <c r="K56" s="62"/>
       <c r="L56" s="14"/>
       <c r="M56" s="19" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B57" s="51"/>
-      <c r="C57" s="58"/>
-      <c r="D57" s="58" t="s">
+      <c r="B57" s="54"/>
+      <c r="C57" s="61"/>
+      <c r="D57" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="E57" s="58"/>
-      <c r="F57" s="58" t="s">
+      <c r="E57" s="61"/>
+      <c r="F57" s="61" t="s">
         <v>153</v>
       </c>
-      <c r="G57" s="58"/>
-      <c r="H57" s="58" t="s">
+      <c r="G57" s="61"/>
+      <c r="H57" s="61" t="s">
         <v>153</v>
       </c>
-      <c r="I57" s="59"/>
-      <c r="J57" s="51"/>
-      <c r="K57" s="59"/>
+      <c r="I57" s="62"/>
+      <c r="J57" s="54"/>
+      <c r="K57" s="62"/>
       <c r="L57" s="14"/>
       <c r="M57" s="19" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="B58" s="51" t="s">
+      <c r="B58" s="54" t="s">
         <v>84</v>
       </c>
       <c r="C58" s="18"/>
-      <c r="D58" s="58" t="s">
+      <c r="D58" s="61" t="s">
         <v>84</v>
       </c>
       <c r="E58" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F58" s="58" t="s">
+      <c r="F58" s="61" t="s">
         <v>84</v>
       </c>
       <c r="G58" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H58" s="58" t="s">
+      <c r="H58" s="61" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="J58" s="51"/>
-      <c r="K58" s="59"/>
+      <c r="J58" s="54"/>
+      <c r="K58" s="62"/>
       <c r="L58" s="14"/>
       <c r="M58" s="19" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="B59" s="51"/>
+      <c r="B59" s="54"/>
       <c r="C59" s="18"/>
-      <c r="D59" s="58"/>
+      <c r="D59" s="61"/>
       <c r="E59" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="F59" s="58"/>
+      <c r="F59" s="61"/>
       <c r="G59" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="H59" s="58"/>
+      <c r="H59" s="61"/>
       <c r="I59" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="J59" s="51"/>
-      <c r="K59" s="59"/>
+      <c r="J59" s="54"/>
+      <c r="K59" s="62"/>
       <c r="L59" s="14"/>
       <c r="M59" s="19" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60" s="7" t="s">
         <v>155</v>
       </c>
       <c r="B60" s="27"/>
-      <c r="C60" s="58" t="s">
+      <c r="C60" s="61" t="s">
         <v>84</v>
       </c>
       <c r="D60" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="E60" s="58" t="s">
+      <c r="E60" s="61" t="s">
         <v>84</v>
       </c>
       <c r="F60" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G60" s="58" t="s">
+      <c r="G60" s="61" t="s">
         <v>84</v>
       </c>
       <c r="H60" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="I60" s="59" t="s">
-        <v>84</v>
-      </c>
-      <c r="J60" s="51"/>
-      <c r="K60" s="59"/>
+      <c r="I60" s="62" t="s">
+        <v>84</v>
+      </c>
+      <c r="J60" s="54"/>
+      <c r="K60" s="62"/>
       <c r="L60" s="13"/>
       <c r="M60" s="19" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="7" t="s">
         <v>162</v>
       </c>
       <c r="B61" s="27"/>
-      <c r="C61" s="56"/>
+      <c r="C61" s="59"/>
       <c r="D61" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="E61" s="56"/>
+      <c r="E61" s="59"/>
       <c r="F61" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G61" s="56"/>
+      <c r="G61" s="59"/>
       <c r="H61" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="I61" s="57"/>
-      <c r="J61" s="55"/>
-      <c r="K61" s="57"/>
+      <c r="I61" s="60"/>
+      <c r="J61" s="58"/>
+      <c r="K61" s="60"/>
       <c r="L61" s="14"/>
       <c r="M61" s="19" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B62" s="52"/>
-      <c r="C62" s="53"/>
-      <c r="D62" s="53"/>
-      <c r="E62" s="53"/>
-      <c r="F62" s="53"/>
-      <c r="G62" s="53"/>
-      <c r="H62" s="53"/>
-      <c r="I62" s="54"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="54"/>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B62" s="55"/>
+      <c r="C62" s="56"/>
+      <c r="D62" s="56"/>
+      <c r="E62" s="56"/>
+      <c r="F62" s="56"/>
+      <c r="G62" s="56"/>
+      <c r="H62" s="56"/>
+      <c r="I62" s="57"/>
+      <c r="J62" s="55"/>
+      <c r="K62" s="57"/>
       <c r="L62" s="14"/>
     </row>
-    <row r="63" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B63" s="55"/>
-      <c r="C63" s="56"/>
-      <c r="D63" s="56"/>
-      <c r="E63" s="56"/>
-      <c r="F63" s="56"/>
-      <c r="G63" s="56"/>
-      <c r="H63" s="56"/>
-      <c r="I63" s="57"/>
-      <c r="J63" s="55"/>
-      <c r="K63" s="57"/>
+      <c r="B63" s="58"/>
+      <c r="C63" s="59"/>
+      <c r="D63" s="59"/>
+      <c r="E63" s="59"/>
+      <c r="F63" s="59"/>
+      <c r="G63" s="59"/>
+      <c r="H63" s="59"/>
+      <c r="I63" s="60"/>
+      <c r="J63" s="58"/>
+      <c r="K63" s="60"/>
       <c r="L63" s="14"/>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="52"/>
-      <c r="C64" s="53"/>
-      <c r="D64" s="53" t="s">
+      <c r="B64" s="55"/>
+      <c r="C64" s="56"/>
+      <c r="D64" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="E64" s="53"/>
-      <c r="F64" s="53"/>
-      <c r="G64" s="53"/>
-      <c r="H64" s="53"/>
-      <c r="I64" s="54"/>
+      <c r="E64" s="56"/>
+      <c r="F64" s="56"/>
+      <c r="G64" s="56"/>
+      <c r="H64" s="56"/>
+      <c r="I64" s="57"/>
       <c r="J64" s="33" t="s">
         <v>81</v>
       </c>
@@ -5104,24 +5187,24 @@
         <v>141</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B65" s="51" t="s">
+      <c r="B65" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C65" s="58"/>
-      <c r="D65" s="58"/>
-      <c r="E65" s="58"/>
-      <c r="F65" s="58" t="s">
+      <c r="C65" s="61"/>
+      <c r="D65" s="61"/>
+      <c r="E65" s="61"/>
+      <c r="F65" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="G65" s="58"/>
-      <c r="H65" s="58" t="s">
+      <c r="G65" s="61"/>
+      <c r="H65" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="I65" s="59"/>
+      <c r="I65" s="62"/>
       <c r="J65" s="18" t="s">
         <v>81</v>
       </c>
@@ -5133,26 +5216,26 @@
         <v>128</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B66" s="51" t="s">
+      <c r="B66" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C66" s="58"/>
-      <c r="D66" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E66" s="58"/>
-      <c r="F66" s="58" t="s">
+      <c r="C66" s="61"/>
+      <c r="D66" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E66" s="61"/>
+      <c r="F66" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="G66" s="58"/>
-      <c r="H66" s="58" t="s">
+      <c r="G66" s="61"/>
+      <c r="H66" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="I66" s="59"/>
+      <c r="I66" s="62"/>
       <c r="J66" s="27" t="s">
         <v>81</v>
       </c>
@@ -5164,26 +5247,26 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="B67" s="51" t="s">
+      <c r="B67" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C67" s="58"/>
-      <c r="D67" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E67" s="58"/>
-      <c r="F67" s="58" t="s">
+      <c r="C67" s="61"/>
+      <c r="D67" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E67" s="61"/>
+      <c r="F67" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="G67" s="58"/>
-      <c r="H67" s="58" t="s">
+      <c r="G67" s="61"/>
+      <c r="H67" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="I67" s="59"/>
+      <c r="I67" s="62"/>
       <c r="J67" s="27" t="s">
         <v>81</v>
       </c>
@@ -5195,7 +5278,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" s="7" t="s">
         <v>61</v>
       </c>
@@ -5216,26 +5299,26 @@
         <v>131</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B69" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C69" s="58"/>
-      <c r="D69" s="58" t="s">
+      <c r="B69" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" s="61"/>
+      <c r="D69" s="61" t="s">
         <v>167</v>
       </c>
-      <c r="E69" s="58"/>
-      <c r="F69" s="58" t="s">
+      <c r="E69" s="61"/>
+      <c r="F69" s="61" t="s">
         <v>83</v>
       </c>
-      <c r="G69" s="58"/>
-      <c r="H69" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="I69" s="59"/>
+      <c r="G69" s="61"/>
+      <c r="H69" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I69" s="62"/>
       <c r="J69" s="27" t="s">
         <v>83</v>
       </c>
@@ -5247,43 +5330,43 @@
         <v>132</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B70" s="52"/>
-      <c r="C70" s="53"/>
-      <c r="D70" s="53"/>
-      <c r="E70" s="53"/>
-      <c r="F70" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="G70" s="53"/>
-      <c r="H70" s="53"/>
-      <c r="I70" s="53"/>
-      <c r="J70" s="53"/>
-      <c r="K70" s="54"/>
+      <c r="B70" s="55"/>
+      <c r="C70" s="56"/>
+      <c r="D70" s="56"/>
+      <c r="E70" s="56"/>
+      <c r="F70" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="G70" s="56"/>
+      <c r="H70" s="56"/>
+      <c r="I70" s="56"/>
+      <c r="J70" s="56"/>
+      <c r="K70" s="57"/>
       <c r="L70" s="14"/>
-      <c r="M70" s="66" t="s">
+      <c r="M70" s="69" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B71" s="51" t="s">
+      <c r="B71" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="C71" s="58"/>
-      <c r="D71" s="58" t="s">
+      <c r="C71" s="61"/>
+      <c r="D71" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="E71" s="58"/>
-      <c r="F71" s="58"/>
-      <c r="G71" s="58"/>
-      <c r="H71" s="58"/>
-      <c r="I71" s="59"/>
+      <c r="E71" s="61"/>
+      <c r="F71" s="61"/>
+      <c r="G71" s="61"/>
+      <c r="H71" s="61"/>
+      <c r="I71" s="62"/>
       <c r="J71" s="27" t="s">
         <v>140</v>
       </c>
@@ -5291,22 +5374,22 @@
         <v>140</v>
       </c>
       <c r="L71" s="14"/>
-      <c r="M71" s="66"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M71" s="69"/>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="B72" s="51"/>
-      <c r="C72" s="58"/>
-      <c r="D72" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E72" s="58"/>
-      <c r="F72" s="58"/>
-      <c r="G72" s="58"/>
-      <c r="H72" s="58"/>
-      <c r="I72" s="59"/>
+      <c r="B72" s="54"/>
+      <c r="C72" s="61"/>
+      <c r="D72" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E72" s="61"/>
+      <c r="F72" s="61"/>
+      <c r="G72" s="61"/>
+      <c r="H72" s="61"/>
+      <c r="I72" s="62"/>
       <c r="J72" s="27"/>
       <c r="K72" s="26"/>
       <c r="L72" s="14"/>
@@ -5314,20 +5397,20 @@
         <v>134</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B73" s="51"/>
-      <c r="C73" s="58"/>
-      <c r="D73" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E73" s="58"/>
-      <c r="F73" s="58"/>
-      <c r="G73" s="58"/>
-      <c r="H73" s="58"/>
-      <c r="I73" s="59"/>
+      <c r="B73" s="54"/>
+      <c r="C73" s="61"/>
+      <c r="D73" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E73" s="61"/>
+      <c r="F73" s="61"/>
+      <c r="G73" s="61"/>
+      <c r="H73" s="61"/>
+      <c r="I73" s="62"/>
       <c r="J73" s="27"/>
       <c r="K73" s="26"/>
       <c r="L73" s="14"/>
@@ -5335,22 +5418,22 @@
         <v>135</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B74" s="55"/>
-      <c r="C74" s="56"/>
-      <c r="D74" s="56"/>
-      <c r="E74" s="56"/>
-      <c r="F74" s="56" t="s">
+      <c r="B74" s="58"/>
+      <c r="C74" s="59"/>
+      <c r="D74" s="59"/>
+      <c r="E74" s="59"/>
+      <c r="F74" s="59" t="s">
         <v>83</v>
       </c>
-      <c r="G74" s="56"/>
-      <c r="H74" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="I74" s="57"/>
+      <c r="G74" s="59"/>
+      <c r="H74" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="I74" s="60"/>
       <c r="J74" s="29" t="s">
         <v>83</v>
       </c>
@@ -5362,26 +5445,26 @@
         <v>133</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B75" s="51" t="s">
-        <v>78</v>
-      </c>
-      <c r="C75" s="58"/>
-      <c r="D75" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E75" s="58"/>
-      <c r="F75" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="G75" s="58"/>
-      <c r="H75" s="58" t="s">
-        <v>78</v>
-      </c>
-      <c r="I75" s="59"/>
+      <c r="B75" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75" s="61"/>
+      <c r="D75" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="E75" s="61"/>
+      <c r="F75" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="G75" s="61"/>
+      <c r="H75" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I75" s="62"/>
       <c r="J75" s="27" t="s">
         <v>83</v>
       </c>
@@ -5393,26 +5476,26 @@
         <v>137</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B76" s="60" t="s">
-        <v>78</v>
-      </c>
-      <c r="C76" s="61"/>
-      <c r="D76" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E76" s="61"/>
-      <c r="F76" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="G76" s="61"/>
-      <c r="H76" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="I76" s="62"/>
+      <c r="B76" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76" s="64"/>
+      <c r="D76" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="E76" s="64"/>
+      <c r="F76" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="G76" s="64"/>
+      <c r="H76" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="I76" s="65"/>
       <c r="J76" s="40" t="s">
         <v>83</v>
       </c>
@@ -5693,15 +5776,1615 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E68BE75-6905-4180-B934-6589799B80CA}">
+  <dimension ref="A1:N72"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="2" max="9" width="9.109375" style="1"/>
+    <col min="10" max="10" width="2.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" style="19" customWidth="1"/>
+    <col min="12" max="12" width="68.6640625" style="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="16"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="66" t="s">
+        <v>179</v>
+      </c>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67" t="s">
+        <v>179</v>
+      </c>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="46" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="N3" s="46" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="N4" s="47" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="N5" s="47" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="33"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="57"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="N6" s="47" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="27"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="N7" s="47" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="29"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" s="48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="39"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="19" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="27"/>
+      <c r="C10" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="27"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="27"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="27"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="27"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="55"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="57"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="54"/>
+      <c r="C16" s="61"/>
+      <c r="D16" s="61"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="61"/>
+      <c r="H16" s="61"/>
+      <c r="I16" s="62"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="27"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="27"/>
+      <c r="C19" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="27"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="19" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" s="27"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="27"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="27"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B25" s="55"/>
+      <c r="C25" s="56"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="56"/>
+      <c r="I25" s="57"/>
+      <c r="J25" s="14"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="58"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
+      <c r="G26" s="59"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="60"/>
+      <c r="J26" s="14"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="55" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="56"/>
+      <c r="D27" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="E27" s="56"/>
+      <c r="F27" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="G27" s="56"/>
+      <c r="H27" s="56"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="19" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="54"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="61"/>
+      <c r="E28" s="61"/>
+      <c r="F28" s="61"/>
+      <c r="G28" s="61"/>
+      <c r="H28" s="61"/>
+      <c r="I28" s="62"/>
+      <c r="J28" s="14"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C29" s="61"/>
+      <c r="D29" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="E29" s="61"/>
+      <c r="F29" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G29" s="61"/>
+      <c r="H29" s="61"/>
+      <c r="I29" s="62"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="54"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="61"/>
+      <c r="F30" s="61"/>
+      <c r="G30" s="61"/>
+      <c r="H30" s="61"/>
+      <c r="I30" s="62"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="54"/>
+      <c r="C31" s="61"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
+      <c r="F31" s="61"/>
+      <c r="G31" s="61"/>
+      <c r="H31" s="61"/>
+      <c r="I31" s="62"/>
+      <c r="J31" s="14"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="58"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="59"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="59"/>
+      <c r="I32" s="60"/>
+      <c r="J32" s="14"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B33" s="55"/>
+      <c r="C33" s="56"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
+      <c r="G33" s="56"/>
+      <c r="H33" s="56"/>
+      <c r="I33" s="57"/>
+      <c r="J33" s="14"/>
+    </row>
+    <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="58"/>
+      <c r="C34" s="59"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+      <c r="G34" s="59"/>
+      <c r="H34" s="59"/>
+      <c r="I34" s="60"/>
+      <c r="J34" s="14"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="69" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" s="27"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="69"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="27"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="26"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="69"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="27"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="26"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="69" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" s="27"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="26"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="69"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" s="27"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="26"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="69"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="27"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="F41" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="26"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B42" s="27"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="26"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="27"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="26"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="19" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B44" s="27"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="26"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="19" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="43" t="s">
+        <v>171</v>
+      </c>
+      <c r="B45" s="27"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="26"/>
+      <c r="J45" s="14"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B46" s="54"/>
+      <c r="C46" s="61"/>
+      <c r="D46" s="61"/>
+      <c r="E46" s="61"/>
+      <c r="F46" s="61"/>
+      <c r="G46" s="61"/>
+      <c r="H46" s="61"/>
+      <c r="I46" s="62"/>
+      <c r="J46" s="14"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47" s="58"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="59"/>
+      <c r="F47" s="59"/>
+      <c r="G47" s="59"/>
+      <c r="H47" s="59"/>
+      <c r="I47" s="60"/>
+      <c r="J47" s="14"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" s="55" t="s">
+        <v>179</v>
+      </c>
+      <c r="C48" s="56"/>
+      <c r="D48" s="56"/>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="57"/>
+      <c r="J48" s="14"/>
+      <c r="K48" s="19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C49" s="61"/>
+      <c r="D49" s="61"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
+      <c r="H49" s="61"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B50" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61"/>
+      <c r="F50" s="61"/>
+      <c r="G50" s="61"/>
+      <c r="H50" s="61"/>
+      <c r="I50" s="62"/>
+      <c r="J50" s="14"/>
+      <c r="K50" s="19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C51" s="61"/>
+      <c r="D51" s="61"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="61"/>
+      <c r="G51" s="61"/>
+      <c r="H51" s="61"/>
+      <c r="I51" s="62"/>
+      <c r="J51" s="14"/>
+      <c r="K51" s="19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A52" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B52" s="54"/>
+      <c r="C52" s="61"/>
+      <c r="D52" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="E52" s="61"/>
+      <c r="F52" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G52" s="61"/>
+      <c r="H52" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="I52" s="62"/>
+      <c r="J52" s="14"/>
+      <c r="K52" s="19" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B53" s="54"/>
+      <c r="C53" s="61"/>
+      <c r="D53" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="E53" s="61"/>
+      <c r="F53" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G53" s="61"/>
+      <c r="H53" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="I53" s="62"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A54" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B54" s="54" t="s">
+        <v>84</v>
+      </c>
+      <c r="C54" s="18"/>
+      <c r="D54" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="E54" s="18"/>
+      <c r="F54" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="G54" s="18"/>
+      <c r="H54" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="I54" s="26"/>
+      <c r="J54" s="14"/>
+      <c r="K54" s="19" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B55" s="54"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="61"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="61"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="61"/>
+      <c r="I55" s="26"/>
+      <c r="J55" s="14"/>
+      <c r="K55" s="19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B56" s="27"/>
+      <c r="C56" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="D56" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E56" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="F56" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="G56" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="H56" s="18"/>
+      <c r="I56" s="62" t="s">
+        <v>84</v>
+      </c>
+      <c r="J56" s="14"/>
+      <c r="K56" s="19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B57" s="27"/>
+      <c r="C57" s="59"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="59"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="59"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="60"/>
+      <c r="J57" s="14"/>
+      <c r="K57" s="19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B58" s="55"/>
+      <c r="C58" s="56"/>
+      <c r="D58" s="56"/>
+      <c r="E58" s="56"/>
+      <c r="F58" s="56"/>
+      <c r="G58" s="56"/>
+      <c r="H58" s="56"/>
+      <c r="I58" s="57"/>
+      <c r="J58" s="14"/>
+    </row>
+    <row r="59" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B59" s="58"/>
+      <c r="C59" s="59"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="59"/>
+      <c r="F59" s="59"/>
+      <c r="G59" s="59"/>
+      <c r="H59" s="59"/>
+      <c r="I59" s="60"/>
+      <c r="J59" s="14"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B60" s="55"/>
+      <c r="C60" s="56"/>
+      <c r="D60" s="56"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="56"/>
+      <c r="G60" s="56"/>
+      <c r="H60" s="56"/>
+      <c r="I60" s="57"/>
+      <c r="J60" s="14"/>
+      <c r="K60" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="L60" s="21"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B61" s="54"/>
+      <c r="C61" s="61"/>
+      <c r="D61" s="61"/>
+      <c r="E61" s="61"/>
+      <c r="F61" s="61"/>
+      <c r="G61" s="61"/>
+      <c r="H61" s="61"/>
+      <c r="I61" s="62"/>
+      <c r="J61" s="14"/>
+      <c r="K61" s="19" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A62" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B62" s="54"/>
+      <c r="C62" s="61"/>
+      <c r="D62" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="E62" s="61"/>
+      <c r="F62" s="61"/>
+      <c r="G62" s="61"/>
+      <c r="H62" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="I62" s="62"/>
+      <c r="J62" s="14"/>
+      <c r="K62" s="19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A63" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B63" s="54"/>
+      <c r="C63" s="61"/>
+      <c r="D63" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="E63" s="61"/>
+      <c r="F63" s="61"/>
+      <c r="G63" s="61"/>
+      <c r="H63" s="61"/>
+      <c r="I63" s="62"/>
+      <c r="J63" s="14"/>
+      <c r="K63" s="19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A64" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" s="27"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+      <c r="F64" s="18"/>
+      <c r="G64" s="18"/>
+      <c r="H64" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="I64" s="62"/>
+      <c r="J64" s="14"/>
+      <c r="K64" s="19" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B65" s="54"/>
+      <c r="C65" s="61"/>
+      <c r="D65" s="61"/>
+      <c r="E65" s="61"/>
+      <c r="F65" s="61"/>
+      <c r="G65" s="61"/>
+      <c r="H65" s="61"/>
+      <c r="I65" s="62"/>
+      <c r="J65" s="14"/>
+      <c r="K65" s="19" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B66" s="55"/>
+      <c r="C66" s="56"/>
+      <c r="D66" s="56" t="s">
+        <v>83</v>
+      </c>
+      <c r="E66" s="56"/>
+      <c r="F66" s="56"/>
+      <c r="G66" s="56"/>
+      <c r="H66" s="56" t="s">
+        <v>84</v>
+      </c>
+      <c r="I66" s="57"/>
+      <c r="J66" s="14"/>
+      <c r="K66" s="69" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B67" s="54"/>
+      <c r="C67" s="61"/>
+      <c r="D67" s="61"/>
+      <c r="E67" s="61"/>
+      <c r="F67" s="61"/>
+      <c r="G67" s="61"/>
+      <c r="H67" s="61"/>
+      <c r="I67" s="62"/>
+      <c r="J67" s="14"/>
+      <c r="K67" s="69"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B68" s="54"/>
+      <c r="C68" s="61"/>
+      <c r="D68" s="61"/>
+      <c r="E68" s="61"/>
+      <c r="F68" s="61"/>
+      <c r="G68" s="61"/>
+      <c r="H68" s="61"/>
+      <c r="I68" s="62"/>
+      <c r="J68" s="14"/>
+      <c r="K68" s="19" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B69" s="54"/>
+      <c r="C69" s="61"/>
+      <c r="D69" s="61"/>
+      <c r="E69" s="61"/>
+      <c r="F69" s="61"/>
+      <c r="G69" s="61"/>
+      <c r="H69" s="61"/>
+      <c r="I69" s="62"/>
+      <c r="J69" s="14"/>
+      <c r="K69" s="19" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B70" s="58"/>
+      <c r="C70" s="59"/>
+      <c r="D70" s="59"/>
+      <c r="E70" s="59"/>
+      <c r="F70" s="59"/>
+      <c r="G70" s="59"/>
+      <c r="H70" s="59"/>
+      <c r="I70" s="60"/>
+      <c r="J70" s="14"/>
+      <c r="K70" s="19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C71" s="61"/>
+      <c r="D71" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="E71" s="61"/>
+      <c r="F71" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="G71" s="61"/>
+      <c r="H71" s="56" t="s">
+        <v>84</v>
+      </c>
+      <c r="I71" s="57"/>
+      <c r="J71" s="14"/>
+      <c r="K71" s="19" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B72" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="C72" s="64"/>
+      <c r="D72" s="64" t="s">
+        <v>179</v>
+      </c>
+      <c r="E72" s="64"/>
+      <c r="F72" s="64" t="s">
+        <v>179</v>
+      </c>
+      <c r="G72" s="64"/>
+      <c r="H72" s="64"/>
+      <c r="I72" s="65"/>
+      <c r="J72" s="14"/>
+      <c r="K72" s="19" t="s">
+        <v>136</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="113">
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="H71:I72"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="H66:I70"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="K66:K67"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="H62:I63"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="I56:I57"/>
+    <mergeCell ref="B58:I59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="K35:K37"/>
+    <mergeCell ref="K38:K40"/>
+    <mergeCell ref="B46:I47"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="B25:I26"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B2:I59 B60:D60 F60 H60 B61:I61 B62:H62 B63:G63 B64:H64 B65:I65 B66:F66 H66 B67:G70 B71:H71 B72:G72">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>$N$3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="G67:G72 H71 H64:H66 E61:E72 G61:G65 I65 H2:H62 B2:D72 F2:F72 E2:E59 G2:G59 I2:I59 I61" xr:uid="{98A2B0C2-9BC5-490F-B97E-4A8CBDDCF29C}">
+      <formula1>$N$3:$N$8</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{D9AC3529-3286-4ABD-96F3-CA04CDC18649}">
+            <xm:f>enums!$A$7</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF008E00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>B2:B3 D2:D3 F2:F3 H2:H3 B4:I5 B6:D6 F6 H6 B7:I14 B15:B16 D15:D16 F15:F16 H15:H16 B17:J24 B25 B27:B28 D27:D28 F27:F28 H27:H28 B29:J29 B31:J31 B33 B35:J45 B46 B48:B54 D52:D53 F52:F54 H52:H54 C54:E54 G54:G55 I54:I55 C55 E55 B56:I56 D57 F57 H57 B57:B58 B60:B63 D60:D63 H61:H62 F61:F63 B64:H64 H65 B65:B72 D65:D72 F65:F72 H71 J2:J16 K8:K9 J27:J28 J48:J57 L60 J60:J65 J67:J72</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{CEDF53AC-6B60-4D6F-A2D9-E663DE3E82C6}">
+            <xm:f>enums!$A$6</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF00DE00"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{9BD8FBE5-E692-4073-9DC7-E639CA0BA304}">
+            <xm:f>enums!$A$5</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFB9FF2D"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{D6F8B74D-5352-4F42-8A0A-FA2607CB3C08}">
+            <xm:f>enums!$A$4</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFBCFF79"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{590521ED-BA1C-4F4A-AE9C-CFF1032672E8}">
+            <xm:f>enums!$A$3</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FF9DE7A8"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{764F74E9-4242-4BB8-9EFF-40A103D121CC}">
+            <xm:f>enums!$A$2</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="6" tint="0.79998168889431442"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{49F21BEC-0B35-4E4C-8F70-B353CF32B028}">
+            <xm:f>enums!$A$8</xm:f>
+            <x14:dxf>
+              <font>
+                <color theme="1" tint="0.34998626667073579"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-0.14996795556505021"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{AEE5FF87-2A9C-4FAC-BC91-3B9C285D3793}">
+            <xm:f>enums!$A$9</xm:f>
+            <x14:dxf>
+              <font>
+                <color auto="1"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="5" tint="0.59996337778862885"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{505ED184-22C4-4943-A7FF-D4B1DD0B9962}">
+            <xm:f>enums!$A$10</xm:f>
+            <x14:dxf>
+              <font>
+                <color auto="1"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor theme="5" tint="0.39994506668294322"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="beginsWith" priority="11" operator="beginsWith" id="{805C8194-5D39-4BDD-8CA8-54F71E8B3AC4}">
+            <xm:f>LEFT(B2,LEN("512"))="512"</xm:f>
+            <xm:f>"512"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="7" tint="0.39994506668294322"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>B2:B3 D2:D3 F2:F3 H2:H3 J2:J16 B4:I5 B6:D6 F6 H6 B7:I14 K8:K9 B15:B16 D15:D16 F15:F16 H15:H16 B17:J24 B25 B27:B28 D27:D28 F27:F28 H27:H28 J27:J28 B29:J29 B31:J31 B33 B35:J45 B46 B48:B54 J48:J57 D52:D53 F52:F54 H52:H54 C54:E54 G54:G55 I54:I55 C55 E55 B56:I56 D57 F57 H57 B57:B58 L60 B60:B63 D60:D63 J60:J65 H61:H62 F61:F63 B64:H64 H65 B65:B72 D65:D72 F65:F72 J67:J72 H71</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{0C526B41-5290-4BD0-8365-CDD66D61BD53}">
+          <x14:formula1>
+            <xm:f>enums!$A$2:$A$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>J67:J72 J2:J65</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42270057-09F5-4DBC-B29A-71117FFFAFC1}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="29.5703125" style="42" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.5546875" style="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="44" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="44" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
         <v>172</v>
       </c>
@@ -5709,67 +7392,67 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>167</v>
       </c>
@@ -5777,7 +7460,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>166</v>
       </c>

</xml_diff>

<commit_message>
Better `cmpGrt_u64` via half-subtractor
- Improves 64-bit compare by replacing implementation with half-subtractor method. Saves on one operation, shorter chain, and 2 less register-register moves.
- Changed 64-bit greater or equal by inlining `cmpLss` so the inversion can be made free.
- Changed the 64-bit saturation addition method to use compare as it is now cheap enough.
- Added 32 and 64-bit average methods. These follow the SSE convention of producing a n+1 bit sum and rounding down.
- Updated the instruction counts and version number to reflect these changes.
</commit_message>
<xml_diff>
--- a/external/InstructionCost.xlsx
+++ b/external/InstructionCost.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\walte\Desktop\Coding\Filling SIMD gaps\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\walte\Documents\GitHub\SSE2-Complete\external\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F29AFA-CAE3-4C54-98C6-4FE8C40F5DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3B7FC7-DAD8-430D-A700-5B86D1F03E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{0228E47D-794C-431C-A2A8-62B0A8D25E03}"/>
+    <workbookView xWindow="38280" yWindow="1605" windowWidth="29040" windowHeight="15840" xr2:uid="{0228E47D-794C-431C-A2A8-62B0A8D25E03}"/>
   </bookViews>
   <sheets>
     <sheet name="Emulated" sheetId="1" r:id="rId1"/>
@@ -2146,7 +2146,7 @@
         <v>13</v>
       </c>
       <c r="I5" s="6">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>36</v>
@@ -2181,7 +2181,7 @@
         <v>13</v>
       </c>
       <c r="I6" s="6">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>36</v>
@@ -2203,9 +2203,13 @@
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
+      <c r="G7" s="1">
+        <v>7</v>
+      </c>
       <c r="H7" s="1"/>
-      <c r="I7" s="6"/>
+      <c r="I7" s="6">
+        <v>7</v>
+      </c>
       <c r="J7" s="1"/>
       <c r="K7" s="6"/>
     </row>
@@ -2904,7 +2908,7 @@
         <v>9</v>
       </c>
       <c r="I30" s="6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J30" s="1">
         <v>1</v>
@@ -2939,7 +2943,7 @@
         <v>9</v>
       </c>
       <c r="I31" s="6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J31" s="1">
         <v>1</v>
@@ -2965,10 +2969,10 @@
         <v>6</v>
       </c>
       <c r="H32" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I32" s="6">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J32" s="1">
         <v>1</v>
@@ -2994,10 +2998,10 @@
         <v>6</v>
       </c>
       <c r="H33" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I33" s="6">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J33" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
Better u8 variable right & arithmetic shifts
- Improved variable 8-bit right shift by replacing `((x >> n) & c) | (x & ~c)` => `max(x << n, (x & ~c))`. Works because shift is smaller.
- Replaced arithmetic shift by constant with alternative method with shorter dependency chain.
</commit_message>
<xml_diff>
--- a/external/InstructionCost.xlsx
+++ b/external/InstructionCost.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\walte\Desktop\Coding\Filling SIMD gaps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A40CC9-772C-4DD6-9812-7D01584470DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0D6475-0F03-43CE-8317-EE64E6D9FB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{0228E47D-794C-431C-A2A8-62B0A8D25E03}"/>
   </bookViews>
@@ -1403,25 +1403,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1430,28 +1436,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1463,8 +1457,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2325,19 +2325,19 @@
       <c r="B11" s="51">
         <v>25</v>
       </c>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52">
+      <c r="C11" s="49"/>
+      <c r="D11" s="49">
         <v>13</v>
       </c>
-      <c r="E11" s="52"/>
-      <c r="F11" s="52">
+      <c r="E11" s="49"/>
+      <c r="F11" s="49">
         <v>12</v>
       </c>
-      <c r="G11" s="52"/>
-      <c r="H11" s="52">
+      <c r="G11" s="49"/>
+      <c r="H11" s="49">
         <v>6</v>
       </c>
-      <c r="I11" s="53"/>
+      <c r="I11" s="50"/>
       <c r="J11" s="1" t="s">
         <v>36</v>
       </c>
@@ -2350,21 +2350,21 @@
         <v>175</v>
       </c>
       <c r="B12" s="51">
-        <v>27</v>
-      </c>
-      <c r="C12" s="52"/>
-      <c r="D12" s="52">
         <v>21</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52">
+      <c r="C12" s="49"/>
+      <c r="D12" s="49">
+        <v>21</v>
+      </c>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49">
         <v>19</v>
       </c>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52">
+      <c r="G12" s="49"/>
+      <c r="H12" s="49">
         <v>6</v>
       </c>
-      <c r="I12" s="53"/>
+      <c r="I12" s="50"/>
       <c r="J12" s="1" t="s">
         <v>36</v>
       </c>
@@ -2379,19 +2379,19 @@
       <c r="B13" s="51">
         <v>86</v>
       </c>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52">
+      <c r="C13" s="49"/>
+      <c r="D13" s="49">
         <v>19</v>
       </c>
-      <c r="E13" s="52"/>
-      <c r="F13" s="52">
+      <c r="E13" s="49"/>
+      <c r="F13" s="49">
         <v>16</v>
       </c>
-      <c r="G13" s="52"/>
-      <c r="H13" s="52">
+      <c r="G13" s="49"/>
+      <c r="H13" s="49">
         <v>9</v>
       </c>
-      <c r="I13" s="53"/>
+      <c r="I13" s="50"/>
       <c r="J13" s="1" t="s">
         <v>36</v>
       </c>
@@ -2553,19 +2553,19 @@
       <c r="B19" s="51">
         <v>7</v>
       </c>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52">
-        <v>1</v>
-      </c>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52">
+      <c r="C19" s="49"/>
+      <c r="D19" s="49">
+        <v>1</v>
+      </c>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49">
         <v>8</v>
       </c>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52">
+      <c r="G19" s="49"/>
+      <c r="H19" s="49">
         <v>13</v>
       </c>
-      <c r="I19" s="53"/>
+      <c r="I19" s="50"/>
       <c r="J19" s="1" t="s">
         <v>36</v>
       </c>
@@ -2712,11 +2712,11 @@
       <c r="K23" s="6">
         <v>1</v>
       </c>
-      <c r="L23" s="49" t="s">
+      <c r="L23" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="53"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
@@ -2740,9 +2740,9 @@
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="6"/>
-      <c r="L24" s="49"/>
-      <c r="M24" s="50"/>
-      <c r="N24" s="50"/>
+      <c r="L24" s="52"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
@@ -2770,9 +2770,9 @@
       <c r="K25" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="L25" s="49"/>
-      <c r="M25" s="50"/>
-      <c r="N25" s="50"/>
+      <c r="L25" s="52"/>
+      <c r="M25" s="53"/>
+      <c r="N25" s="53"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
@@ -2796,9 +2796,9 @@
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="6"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="50"/>
-      <c r="N26" s="50"/>
+      <c r="L26" s="52"/>
+      <c r="M26" s="53"/>
+      <c r="N26" s="53"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
@@ -2874,19 +2874,19 @@
       <c r="B29" s="51">
         <v>1</v>
       </c>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52">
-        <v>1</v>
-      </c>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52">
-        <v>1</v>
-      </c>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52">
+      <c r="C29" s="49"/>
+      <c r="D29" s="49">
+        <v>1</v>
+      </c>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49">
+        <v>1</v>
+      </c>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49">
         <v>3</v>
       </c>
-      <c r="I29" s="53"/>
+      <c r="I29" s="50"/>
       <c r="J29" s="1">
         <v>1</v>
       </c>
@@ -3369,6 +3369,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="L23:N26"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="H19:I19"/>
@@ -3385,11 +3390,6 @@
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="H13:I13"/>
-    <mergeCell ref="L23:N26"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:C11 B12:K12 B13 D13 B14:K26 B3:K10 F11:K11 F13 H13 J13:K13 B29:K33 B36:K43">
     <cfRule type="containsBlanks" dxfId="22" priority="12">
@@ -3481,22 +3481,22 @@
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="66" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67" t="s">
-        <v>78</v>
-      </c>
-      <c r="I2" s="68"/>
+      <c r="B2" s="64" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="I2" s="66"/>
       <c r="J2" s="31" t="s">
         <v>83</v>
       </c>
@@ -3515,19 +3515,19 @@
       <c r="B3" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="I3" s="62"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" s="55"/>
       <c r="J3" s="27" t="s">
         <v>83</v>
       </c>
@@ -3607,18 +3607,18 @@
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34"/>
-      <c r="D6" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56" t="s">
+      <c r="D6" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56" t="s">
+      <c r="G6" s="58"/>
+      <c r="H6" s="58" t="s">
         <v>167</v>
       </c>
-      <c r="I6" s="57"/>
+      <c r="I6" s="59"/>
       <c r="J6" s="33" t="s">
         <v>84</v>
       </c>
@@ -3948,18 +3948,18 @@
       <c r="A17" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="55"/>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56" t="s">
+      <c r="B17" s="63"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56" t="s">
+      <c r="E17" s="58"/>
+      <c r="F17" s="58" t="s">
         <v>80</v>
       </c>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="57"/>
+      <c r="G17" s="58"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="59"/>
       <c r="J17" s="33" t="s">
         <v>79</v>
       </c>
@@ -3976,17 +3976,17 @@
         <v>58</v>
       </c>
       <c r="B18" s="54"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61" t="s">
+      <c r="C18" s="60"/>
+      <c r="D18" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61" t="s">
+      <c r="E18" s="60"/>
+      <c r="F18" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="62"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="60"/>
+      <c r="I18" s="55"/>
       <c r="J18" s="27" t="s">
         <v>79</v>
       </c>
@@ -4267,54 +4267,54 @@
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B29" s="55"/>
-      <c r="C29" s="56"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="55"/>
-      <c r="K29" s="57"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="63"/>
+      <c r="K29" s="59"/>
       <c r="L29" s="14"/>
     </row>
     <row r="30" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="58"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="59"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="59"/>
-      <c r="H30" s="59"/>
-      <c r="I30" s="60"/>
-      <c r="J30" s="58"/>
-      <c r="K30" s="60"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="61"/>
+      <c r="F30" s="61"/>
+      <c r="G30" s="61"/>
+      <c r="H30" s="61"/>
+      <c r="I30" s="57"/>
+      <c r="J30" s="56"/>
+      <c r="K30" s="57"/>
       <c r="L30" s="14"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="55" t="s">
-        <v>78</v>
-      </c>
-      <c r="C31" s="56"/>
-      <c r="D31" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="E31" s="56"/>
-      <c r="F31" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="G31" s="56"/>
-      <c r="H31" s="56" t="s">
+      <c r="B31" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="58"/>
+      <c r="D31" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="E31" s="58"/>
+      <c r="F31" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="G31" s="58"/>
+      <c r="H31" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="I31" s="57"/>
+      <c r="I31" s="59"/>
       <c r="J31" s="33" t="s">
         <v>83</v>
       </c>
@@ -4333,19 +4333,19 @@
       <c r="B32" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61" t="s">
+      <c r="C32" s="60"/>
+      <c r="D32" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="E32" s="61"/>
-      <c r="F32" s="61" t="s">
+      <c r="E32" s="60"/>
+      <c r="F32" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61" t="s">
+      <c r="G32" s="60"/>
+      <c r="H32" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="I32" s="62"/>
+      <c r="I32" s="55"/>
       <c r="J32" s="27" t="s">
         <v>83</v>
       </c>
@@ -4361,31 +4361,31 @@
       <c r="B33" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="61" t="s">
+      <c r="C33" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="D33" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E33" s="61" t="s">
+      <c r="D33" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E33" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="F33" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="G33" s="61" t="s">
+      <c r="F33" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G33" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="H33" s="61" t="s">
+      <c r="H33" s="60" t="s">
         <v>82</v>
       </c>
-      <c r="I33" s="62" t="s">
+      <c r="I33" s="55" t="s">
         <v>167</v>
       </c>
       <c r="J33" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="K33" s="62" t="s">
+      <c r="K33" s="55" t="s">
         <v>78</v>
       </c>
       <c r="L33" s="18"/>
@@ -4398,15 +4398,15 @@
         <v>50</v>
       </c>
       <c r="B34" s="54"/>
-      <c r="C34" s="61"/>
-      <c r="D34" s="61"/>
-      <c r="E34" s="61"/>
-      <c r="F34" s="61"/>
-      <c r="G34" s="61"/>
-      <c r="H34" s="61"/>
-      <c r="I34" s="62"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="60"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="60"/>
+      <c r="I34" s="55"/>
       <c r="J34" s="54"/>
-      <c r="K34" s="62"/>
+      <c r="K34" s="55"/>
       <c r="L34" s="18"/>
       <c r="M34" s="19" t="s">
         <v>118</v>
@@ -4419,31 +4419,31 @@
       <c r="B35" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="C35" s="61" t="s">
+      <c r="C35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="D35" s="61" t="s">
+      <c r="D35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="E35" s="61" t="s">
+      <c r="E35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="F35" s="61" t="s">
+      <c r="F35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="G35" s="61" t="s">
+      <c r="G35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="H35" s="61" t="s">
+      <c r="H35" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="I35" s="62" t="s">
+      <c r="I35" s="55" t="s">
         <v>167</v>
       </c>
       <c r="J35" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="K35" s="62" t="s">
+      <c r="K35" s="55" t="s">
         <v>78</v>
       </c>
       <c r="L35" s="14"/>
@@ -4452,45 +4452,45 @@
       <c r="A36" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="58"/>
-      <c r="C36" s="59"/>
-      <c r="D36" s="59"/>
-      <c r="E36" s="59"/>
-      <c r="F36" s="59"/>
-      <c r="G36" s="59"/>
-      <c r="H36" s="59"/>
-      <c r="I36" s="60"/>
-      <c r="J36" s="58"/>
-      <c r="K36" s="60"/>
+      <c r="B36" s="56"/>
+      <c r="C36" s="61"/>
+      <c r="D36" s="61"/>
+      <c r="E36" s="61"/>
+      <c r="F36" s="61"/>
+      <c r="G36" s="61"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="57"/>
+      <c r="J36" s="56"/>
+      <c r="K36" s="57"/>
       <c r="L36" s="14"/>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B37" s="55"/>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="57"/>
-      <c r="J37" s="55"/>
-      <c r="K37" s="57"/>
+      <c r="B37" s="63"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="59"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="59"/>
       <c r="L37" s="14"/>
     </row>
     <row r="38" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B38" s="58"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="59"/>
-      <c r="H38" s="59"/>
-      <c r="I38" s="60"/>
-      <c r="J38" s="58"/>
-      <c r="K38" s="60"/>
+      <c r="B38" s="56"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="57"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="57"/>
       <c r="L38" s="14"/>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
@@ -4528,7 +4528,7 @@
         <v>84</v>
       </c>
       <c r="L39" s="14"/>
-      <c r="M39" s="69" t="s">
+      <c r="M39" s="62" t="s">
         <v>119</v>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
         <v>84</v>
       </c>
       <c r="L40" s="14"/>
-      <c r="M40" s="69"/>
+      <c r="M40" s="62"/>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
@@ -4604,7 +4604,7 @@
         <v>84</v>
       </c>
       <c r="L41" s="14"/>
-      <c r="M41" s="69"/>
+      <c r="M41" s="62"/>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
@@ -4641,7 +4641,7 @@
         <v>84</v>
       </c>
       <c r="L42" s="14"/>
-      <c r="M42" s="69" t="s">
+      <c r="M42" s="62" t="s">
         <v>120</v>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
         <v>84</v>
       </c>
       <c r="L43" s="14"/>
-      <c r="M43" s="69"/>
+      <c r="M43" s="62"/>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
@@ -4717,7 +4717,7 @@
         <v>84</v>
       </c>
       <c r="L44" s="14"/>
-      <c r="M44" s="69"/>
+      <c r="M44" s="62"/>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
@@ -4855,47 +4855,47 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B50" s="54"/>
-      <c r="C50" s="61"/>
-      <c r="D50" s="61"/>
-      <c r="E50" s="61"/>
-      <c r="F50" s="61"/>
-      <c r="G50" s="61"/>
-      <c r="H50" s="61"/>
-      <c r="I50" s="62"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="60"/>
+      <c r="E50" s="60"/>
+      <c r="F50" s="60"/>
+      <c r="G50" s="60"/>
+      <c r="H50" s="60"/>
+      <c r="I50" s="55"/>
       <c r="J50" s="54"/>
-      <c r="K50" s="62"/>
+      <c r="K50" s="55"/>
       <c r="L50" s="14"/>
     </row>
     <row r="51" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B51" s="58"/>
-      <c r="C51" s="59"/>
-      <c r="D51" s="59"/>
-      <c r="E51" s="59"/>
-      <c r="F51" s="59"/>
-      <c r="G51" s="59"/>
-      <c r="H51" s="59"/>
-      <c r="I51" s="60"/>
-      <c r="J51" s="58"/>
-      <c r="K51" s="60"/>
+      <c r="B51" s="56"/>
+      <c r="C51" s="61"/>
+      <c r="D51" s="61"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="61"/>
+      <c r="G51" s="61"/>
+      <c r="H51" s="61"/>
+      <c r="I51" s="57"/>
+      <c r="J51" s="56"/>
+      <c r="K51" s="57"/>
       <c r="L51" s="14"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B52" s="55" t="s">
-        <v>78</v>
-      </c>
-      <c r="C52" s="56"/>
-      <c r="D52" s="56"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="56"/>
-      <c r="G52" s="56"/>
-      <c r="H52" s="56"/>
-      <c r="I52" s="57"/>
+      <c r="B52" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" s="58"/>
+      <c r="D52" s="58"/>
+      <c r="E52" s="58"/>
+      <c r="F52" s="58"/>
+      <c r="G52" s="58"/>
+      <c r="H52" s="58"/>
+      <c r="I52" s="59"/>
       <c r="J52" s="33" t="s">
         <v>83</v>
       </c>
@@ -4914,13 +4914,13 @@
       <c r="B53" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C53" s="61"/>
-      <c r="D53" s="61"/>
-      <c r="E53" s="61"/>
-      <c r="F53" s="61"/>
-      <c r="G53" s="61"/>
-      <c r="H53" s="61"/>
-      <c r="I53" s="62"/>
+      <c r="C53" s="60"/>
+      <c r="D53" s="60"/>
+      <c r="E53" s="60"/>
+      <c r="F53" s="60"/>
+      <c r="G53" s="60"/>
+      <c r="H53" s="60"/>
+      <c r="I53" s="55"/>
       <c r="J53" s="27" t="s">
         <v>83</v>
       </c>
@@ -4939,13 +4939,13 @@
       <c r="B54" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C54" s="61"/>
-      <c r="D54" s="61"/>
-      <c r="E54" s="61"/>
-      <c r="F54" s="61"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="61"/>
-      <c r="I54" s="62"/>
+      <c r="C54" s="60"/>
+      <c r="D54" s="60"/>
+      <c r="E54" s="60"/>
+      <c r="F54" s="60"/>
+      <c r="G54" s="60"/>
+      <c r="H54" s="60"/>
+      <c r="I54" s="55"/>
       <c r="J54" s="27" t="s">
         <v>83</v>
       </c>
@@ -4964,13 +4964,13 @@
       <c r="B55" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C55" s="61"/>
-      <c r="D55" s="61"/>
-      <c r="E55" s="61"/>
-      <c r="F55" s="61"/>
-      <c r="G55" s="61"/>
-      <c r="H55" s="61"/>
-      <c r="I55" s="62"/>
+      <c r="C55" s="60"/>
+      <c r="D55" s="60"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="60"/>
+      <c r="G55" s="60"/>
+      <c r="H55" s="60"/>
+      <c r="I55" s="55"/>
       <c r="J55" s="27" t="s">
         <v>83</v>
       </c>
@@ -4987,23 +4987,23 @@
         <v>158</v>
       </c>
       <c r="B56" s="54"/>
-      <c r="C56" s="61"/>
-      <c r="D56" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E56" s="61"/>
-      <c r="F56" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="G56" s="61"/>
-      <c r="H56" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="I56" s="62"/>
+      <c r="C56" s="60"/>
+      <c r="D56" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E56" s="60"/>
+      <c r="F56" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G56" s="60"/>
+      <c r="H56" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="I56" s="55"/>
       <c r="J56" s="54" t="s">
         <v>84</v>
       </c>
-      <c r="K56" s="62"/>
+      <c r="K56" s="55"/>
       <c r="L56" s="14"/>
       <c r="M56" s="19" t="s">
         <v>124</v>
@@ -5014,21 +5014,21 @@
         <v>157</v>
       </c>
       <c r="B57" s="54"/>
-      <c r="C57" s="61"/>
-      <c r="D57" s="61" t="s">
+      <c r="C57" s="60"/>
+      <c r="D57" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="E57" s="61"/>
-      <c r="F57" s="61" t="s">
+      <c r="E57" s="60"/>
+      <c r="F57" s="60" t="s">
         <v>153</v>
       </c>
-      <c r="G57" s="61"/>
-      <c r="H57" s="61" t="s">
+      <c r="G57" s="60"/>
+      <c r="H57" s="60" t="s">
         <v>153</v>
       </c>
-      <c r="I57" s="62"/>
+      <c r="I57" s="55"/>
       <c r="J57" s="54"/>
-      <c r="K57" s="62"/>
+      <c r="K57" s="55"/>
       <c r="L57" s="14"/>
       <c r="M57" s="19" t="s">
         <v>159</v>
@@ -5042,26 +5042,26 @@
         <v>84</v>
       </c>
       <c r="C58" s="18"/>
-      <c r="D58" s="61" t="s">
+      <c r="D58" s="60" t="s">
         <v>84</v>
       </c>
       <c r="E58" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F58" s="61" t="s">
+      <c r="F58" s="60" t="s">
         <v>84</v>
       </c>
       <c r="G58" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="H58" s="61" t="s">
+      <c r="H58" s="60" t="s">
         <v>84</v>
       </c>
       <c r="I58" s="18" t="s">
         <v>78</v>
       </c>
       <c r="J58" s="54"/>
-      <c r="K58" s="62"/>
+      <c r="K58" s="55"/>
       <c r="L58" s="14"/>
       <c r="M58" s="19" t="s">
         <v>125</v>
@@ -5073,20 +5073,20 @@
       </c>
       <c r="B59" s="54"/>
       <c r="C59" s="18"/>
-      <c r="D59" s="61"/>
+      <c r="D59" s="60"/>
       <c r="E59" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="F59" s="61"/>
+      <c r="F59" s="60"/>
       <c r="G59" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="H59" s="61"/>
+      <c r="H59" s="60"/>
       <c r="I59" s="18" t="s">
         <v>153</v>
       </c>
       <c r="J59" s="54"/>
-      <c r="K59" s="62"/>
+      <c r="K59" s="55"/>
       <c r="L59" s="14"/>
       <c r="M59" s="19" t="s">
         <v>160</v>
@@ -5097,29 +5097,29 @@
         <v>155</v>
       </c>
       <c r="B60" s="27"/>
-      <c r="C60" s="61" t="s">
+      <c r="C60" s="60" t="s">
         <v>84</v>
       </c>
       <c r="D60" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="E60" s="61" t="s">
+      <c r="E60" s="60" t="s">
         <v>84</v>
       </c>
       <c r="F60" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G60" s="61" t="s">
+      <c r="G60" s="60" t="s">
         <v>84</v>
       </c>
       <c r="H60" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="I60" s="62" t="s">
+      <c r="I60" s="55" t="s">
         <v>84</v>
       </c>
       <c r="J60" s="54"/>
-      <c r="K60" s="62"/>
+      <c r="K60" s="55"/>
       <c r="L60" s="13"/>
       <c r="M60" s="19" t="s">
         <v>126</v>
@@ -5130,69 +5130,69 @@
         <v>162</v>
       </c>
       <c r="B61" s="27"/>
-      <c r="C61" s="59"/>
+      <c r="C61" s="61"/>
       <c r="D61" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="E61" s="59"/>
+      <c r="E61" s="61"/>
       <c r="F61" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G61" s="59"/>
+      <c r="G61" s="61"/>
       <c r="H61" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="I61" s="60"/>
-      <c r="J61" s="58"/>
-      <c r="K61" s="60"/>
+      <c r="I61" s="57"/>
+      <c r="J61" s="56"/>
+      <c r="K61" s="57"/>
       <c r="L61" s="14"/>
       <c r="M61" s="19" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B62" s="55"/>
-      <c r="C62" s="56"/>
-      <c r="D62" s="56"/>
-      <c r="E62" s="56"/>
-      <c r="F62" s="56"/>
-      <c r="G62" s="56"/>
-      <c r="H62" s="56"/>
-      <c r="I62" s="57"/>
-      <c r="J62" s="55"/>
-      <c r="K62" s="57"/>
+      <c r="B62" s="63"/>
+      <c r="C62" s="58"/>
+      <c r="D62" s="58"/>
+      <c r="E62" s="58"/>
+      <c r="F62" s="58"/>
+      <c r="G62" s="58"/>
+      <c r="H62" s="58"/>
+      <c r="I62" s="59"/>
+      <c r="J62" s="63"/>
+      <c r="K62" s="59"/>
       <c r="L62" s="14"/>
     </row>
     <row r="63" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B63" s="58"/>
-      <c r="C63" s="59"/>
-      <c r="D63" s="59"/>
-      <c r="E63" s="59"/>
-      <c r="F63" s="59"/>
-      <c r="G63" s="59"/>
-      <c r="H63" s="59"/>
-      <c r="I63" s="60"/>
-      <c r="J63" s="58"/>
-      <c r="K63" s="60"/>
+      <c r="B63" s="56"/>
+      <c r="C63" s="61"/>
+      <c r="D63" s="61"/>
+      <c r="E63" s="61"/>
+      <c r="F63" s="61"/>
+      <c r="G63" s="61"/>
+      <c r="H63" s="61"/>
+      <c r="I63" s="57"/>
+      <c r="J63" s="56"/>
+      <c r="K63" s="57"/>
       <c r="L63" s="14"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B64" s="55"/>
-      <c r="C64" s="56"/>
-      <c r="D64" s="56" t="s">
+      <c r="B64" s="63"/>
+      <c r="C64" s="58"/>
+      <c r="D64" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="E64" s="56"/>
-      <c r="F64" s="56"/>
-      <c r="G64" s="56"/>
-      <c r="H64" s="56"/>
-      <c r="I64" s="57"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="58"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="58"/>
+      <c r="I64" s="59"/>
       <c r="J64" s="33" t="s">
         <v>81</v>
       </c>
@@ -5214,17 +5214,17 @@
       <c r="B65" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C65" s="61"/>
-      <c r="D65" s="61"/>
-      <c r="E65" s="61"/>
-      <c r="F65" s="61" t="s">
+      <c r="C65" s="60"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="60"/>
+      <c r="F65" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="G65" s="61"/>
-      <c r="H65" s="61" t="s">
+      <c r="G65" s="60"/>
+      <c r="H65" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="I65" s="62"/>
+      <c r="I65" s="55"/>
       <c r="J65" s="18" t="s">
         <v>81</v>
       </c>
@@ -5243,19 +5243,19 @@
       <c r="B66" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C66" s="61"/>
-      <c r="D66" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E66" s="61"/>
-      <c r="F66" s="61" t="s">
+      <c r="C66" s="60"/>
+      <c r="D66" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E66" s="60"/>
+      <c r="F66" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="G66" s="61"/>
-      <c r="H66" s="61" t="s">
+      <c r="G66" s="60"/>
+      <c r="H66" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="I66" s="62"/>
+      <c r="I66" s="55"/>
       <c r="J66" s="27" t="s">
         <v>81</v>
       </c>
@@ -5274,19 +5274,19 @@
       <c r="B67" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="C67" s="61"/>
-      <c r="D67" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E67" s="61"/>
-      <c r="F67" s="61" t="s">
+      <c r="C67" s="60"/>
+      <c r="D67" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E67" s="60"/>
+      <c r="F67" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="G67" s="61"/>
-      <c r="H67" s="61" t="s">
+      <c r="G67" s="60"/>
+      <c r="H67" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="I67" s="62"/>
+      <c r="I67" s="55"/>
       <c r="J67" s="27" t="s">
         <v>81</v>
       </c>
@@ -5326,19 +5326,19 @@
       <c r="B69" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C69" s="61"/>
-      <c r="D69" s="61" t="s">
+      <c r="C69" s="60"/>
+      <c r="D69" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="E69" s="61"/>
-      <c r="F69" s="61" t="s">
+      <c r="E69" s="60"/>
+      <c r="F69" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="G69" s="61"/>
-      <c r="H69" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="I69" s="62"/>
+      <c r="G69" s="60"/>
+      <c r="H69" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="I69" s="55"/>
       <c r="J69" s="27" t="s">
         <v>83</v>
       </c>
@@ -5354,20 +5354,20 @@
       <c r="A70" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B70" s="55"/>
-      <c r="C70" s="56"/>
-      <c r="D70" s="56"/>
-      <c r="E70" s="56"/>
-      <c r="F70" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="G70" s="56"/>
-      <c r="H70" s="56"/>
-      <c r="I70" s="56"/>
-      <c r="J70" s="56"/>
-      <c r="K70" s="57"/>
+      <c r="B70" s="63"/>
+      <c r="C70" s="58"/>
+      <c r="D70" s="58"/>
+      <c r="E70" s="58"/>
+      <c r="F70" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="G70" s="58"/>
+      <c r="H70" s="58"/>
+      <c r="I70" s="58"/>
+      <c r="J70" s="58"/>
+      <c r="K70" s="59"/>
       <c r="L70" s="14"/>
-      <c r="M70" s="69" t="s">
+      <c r="M70" s="62" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5378,15 +5378,15 @@
       <c r="B71" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="C71" s="61"/>
-      <c r="D71" s="61" t="s">
+      <c r="C71" s="60"/>
+      <c r="D71" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="E71" s="61"/>
-      <c r="F71" s="61"/>
-      <c r="G71" s="61"/>
-      <c r="H71" s="61"/>
-      <c r="I71" s="62"/>
+      <c r="E71" s="60"/>
+      <c r="F71" s="60"/>
+      <c r="G71" s="60"/>
+      <c r="H71" s="60"/>
+      <c r="I71" s="55"/>
       <c r="J71" s="27" t="s">
         <v>140</v>
       </c>
@@ -5394,22 +5394,22 @@
         <v>140</v>
       </c>
       <c r="L71" s="14"/>
-      <c r="M71" s="69"/>
+      <c r="M71" s="62"/>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" s="7" t="s">
         <v>143</v>
       </c>
       <c r="B72" s="54"/>
-      <c r="C72" s="61"/>
-      <c r="D72" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E72" s="61"/>
-      <c r="F72" s="61"/>
-      <c r="G72" s="61"/>
-      <c r="H72" s="61"/>
-      <c r="I72" s="62"/>
+      <c r="C72" s="60"/>
+      <c r="D72" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E72" s="60"/>
+      <c r="F72" s="60"/>
+      <c r="G72" s="60"/>
+      <c r="H72" s="60"/>
+      <c r="I72" s="55"/>
       <c r="J72" s="27"/>
       <c r="K72" s="26"/>
       <c r="L72" s="14"/>
@@ -5422,15 +5422,15 @@
         <v>142</v>
       </c>
       <c r="B73" s="54"/>
-      <c r="C73" s="61"/>
-      <c r="D73" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E73" s="61"/>
-      <c r="F73" s="61"/>
-      <c r="G73" s="61"/>
-      <c r="H73" s="61"/>
-      <c r="I73" s="62"/>
+      <c r="C73" s="60"/>
+      <c r="D73" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E73" s="60"/>
+      <c r="F73" s="60"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="60"/>
+      <c r="I73" s="55"/>
       <c r="J73" s="27"/>
       <c r="K73" s="26"/>
       <c r="L73" s="14"/>
@@ -5442,18 +5442,18 @@
       <c r="A74" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B74" s="58"/>
-      <c r="C74" s="59"/>
-      <c r="D74" s="59"/>
-      <c r="E74" s="59"/>
-      <c r="F74" s="59" t="s">
+      <c r="B74" s="56"/>
+      <c r="C74" s="61"/>
+      <c r="D74" s="61"/>
+      <c r="E74" s="61"/>
+      <c r="F74" s="61" t="s">
         <v>83</v>
       </c>
-      <c r="G74" s="59"/>
-      <c r="H74" s="59" t="s">
-        <v>78</v>
-      </c>
-      <c r="I74" s="60"/>
+      <c r="G74" s="61"/>
+      <c r="H74" s="61" t="s">
+        <v>78</v>
+      </c>
+      <c r="I74" s="57"/>
       <c r="J74" s="29" t="s">
         <v>83</v>
       </c>
@@ -5472,19 +5472,19 @@
       <c r="B75" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="C75" s="61"/>
-      <c r="D75" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E75" s="61"/>
-      <c r="F75" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="G75" s="61"/>
-      <c r="H75" s="61" t="s">
-        <v>78</v>
-      </c>
-      <c r="I75" s="62"/>
+      <c r="C75" s="60"/>
+      <c r="D75" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="E75" s="60"/>
+      <c r="F75" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="G75" s="60"/>
+      <c r="H75" s="60" t="s">
+        <v>78</v>
+      </c>
+      <c r="I75" s="55"/>
       <c r="J75" s="27" t="s">
         <v>83</v>
       </c>
@@ -5500,22 +5500,22 @@
       <c r="A76" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B76" s="63" t="s">
-        <v>78</v>
-      </c>
-      <c r="C76" s="64"/>
-      <c r="D76" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="E76" s="64"/>
-      <c r="F76" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="G76" s="64"/>
-      <c r="H76" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I76" s="65"/>
+      <c r="B76" s="67" t="s">
+        <v>78</v>
+      </c>
+      <c r="C76" s="68"/>
+      <c r="D76" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="E76" s="68"/>
+      <c r="F76" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="G76" s="68"/>
+      <c r="H76" s="68" t="s">
+        <v>78</v>
+      </c>
+      <c r="I76" s="69"/>
       <c r="J76" s="40" t="s">
         <v>83</v>
       </c>
@@ -5529,6 +5529,106 @@
     </row>
   </sheetData>
   <mergeCells count="124">
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="B29:I30"/>
+    <mergeCell ref="J29:K30"/>
+    <mergeCell ref="B37:I38"/>
+    <mergeCell ref="J37:K38"/>
+    <mergeCell ref="B50:I51"/>
+    <mergeCell ref="J50:K51"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="H76:I76"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="H74:I74"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="D73:E73"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="H73:I73"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="H75:I75"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="H72:I72"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="H69:I69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="F70:K70"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="M39:M41"/>
+    <mergeCell ref="M42:M44"/>
+    <mergeCell ref="M70:M71"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J62:K63"/>
+    <mergeCell ref="B54:I54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="H66:I66"/>
+    <mergeCell ref="D64:I64"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B62:I63"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="F58:F59"/>
+    <mergeCell ref="H58:H59"/>
     <mergeCell ref="J56:K61"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="B71:C71"/>
@@ -5553,106 +5653,6 @@
     <mergeCell ref="D67:E67"/>
     <mergeCell ref="F67:G67"/>
     <mergeCell ref="H67:I67"/>
-    <mergeCell ref="M39:M41"/>
-    <mergeCell ref="M42:M44"/>
-    <mergeCell ref="M70:M71"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="J62:K63"/>
-    <mergeCell ref="B54:I54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="H66:I66"/>
-    <mergeCell ref="D64:I64"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B62:I63"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="F58:F59"/>
-    <mergeCell ref="H58:H59"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="H65:I65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="H56:I56"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B53:I53"/>
-    <mergeCell ref="I33:I34"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="H72:I72"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="H69:I69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="F70:K70"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="H76:I76"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="H74:I74"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="D75:E75"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="H75:I75"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="B29:I30"/>
-    <mergeCell ref="J29:K30"/>
-    <mergeCell ref="B37:I38"/>
-    <mergeCell ref="J37:K38"/>
-    <mergeCell ref="B50:I51"/>
-    <mergeCell ref="J50:K51"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="B32:C32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5841,20 +5841,20 @@
       <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="64" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67" t="s">
+      <c r="C2" s="65"/>
+      <c r="D2" s="65" t="s">
         <v>179</v>
       </c>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67" t="s">
+      <c r="E2" s="65"/>
+      <c r="F2" s="65" t="s">
         <v>179</v>
       </c>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="68"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="66"/>
       <c r="J2" s="14"/>
       <c r="K2" s="19" t="s">
         <v>10</v>
@@ -5870,17 +5870,17 @@
       <c r="B3" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61" t="s">
+      <c r="C3" s="60"/>
+      <c r="D3" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="E3" s="61"/>
-      <c r="F3" s="61" t="s">
+      <c r="E3" s="60"/>
+      <c r="F3" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="G3" s="61"/>
-      <c r="H3" s="61"/>
-      <c r="I3" s="62"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="55"/>
       <c r="J3" s="14"/>
       <c r="K3" s="19" t="s">
         <v>11</v>
@@ -5951,14 +5951,14 @@
       </c>
       <c r="B6" s="33"/>
       <c r="C6" s="34"/>
-      <c r="D6" s="56" t="s">
+      <c r="D6" s="58" t="s">
         <v>179</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="57"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="59"/>
       <c r="J6" s="14"/>
       <c r="K6" s="19" t="s">
         <v>98</v>
@@ -6121,14 +6121,14 @@
       <c r="A15" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="56"/>
-      <c r="D15" s="56"/>
-      <c r="E15" s="56"/>
-      <c r="F15" s="56"/>
-      <c r="G15" s="56"/>
-      <c r="H15" s="56"/>
-      <c r="I15" s="57"/>
+      <c r="B15" s="63"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="59"/>
       <c r="J15" s="14"/>
       <c r="K15" s="19" t="s">
         <v>104</v>
@@ -6139,13 +6139,13 @@
         <v>58</v>
       </c>
       <c r="B16" s="54"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="61"/>
-      <c r="E16" s="61"/>
-      <c r="F16" s="61"/>
-      <c r="G16" s="61"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="62"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
+      <c r="I16" s="55"/>
       <c r="J16" s="14"/>
       <c r="K16" s="19" t="s">
         <v>105</v>
@@ -6290,48 +6290,48 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B25" s="55"/>
-      <c r="C25" s="56"/>
-      <c r="D25" s="56"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="56"/>
-      <c r="H25" s="56"/>
-      <c r="I25" s="57"/>
+      <c r="B25" s="63"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="59"/>
       <c r="J25" s="14"/>
     </row>
     <row r="26" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="58"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="59"/>
-      <c r="H26" s="59"/>
-      <c r="I26" s="60"/>
+      <c r="B26" s="56"/>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="57"/>
       <c r="J26" s="14"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="55" t="s">
+      <c r="B27" s="63" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="56" t="s">
+      <c r="C27" s="58"/>
+      <c r="D27" s="58" t="s">
         <v>179</v>
       </c>
-      <c r="E27" s="56"/>
-      <c r="F27" s="56" t="s">
+      <c r="E27" s="58"/>
+      <c r="F27" s="58" t="s">
         <v>179</v>
       </c>
-      <c r="G27" s="56"/>
-      <c r="H27" s="56"/>
-      <c r="I27" s="57"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="59"/>
       <c r="J27" s="14"/>
       <c r="K27" s="19" t="s">
         <v>116</v>
@@ -6342,13 +6342,13 @@
         <v>53</v>
       </c>
       <c r="B28" s="54"/>
-      <c r="C28" s="61"/>
-      <c r="D28" s="61"/>
-      <c r="E28" s="61"/>
-      <c r="F28" s="61"/>
-      <c r="G28" s="61"/>
-      <c r="H28" s="61"/>
-      <c r="I28" s="62"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="60"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="60"/>
+      <c r="G28" s="60"/>
+      <c r="H28" s="60"/>
+      <c r="I28" s="55"/>
       <c r="J28" s="14"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
@@ -6358,17 +6358,17 @@
       <c r="B29" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C29" s="61"/>
-      <c r="D29" s="61" t="s">
+      <c r="C29" s="60"/>
+      <c r="D29" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="E29" s="61"/>
-      <c r="F29" s="61" t="s">
+      <c r="E29" s="60"/>
+      <c r="F29" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="G29" s="61"/>
-      <c r="H29" s="61"/>
-      <c r="I29" s="62"/>
+      <c r="G29" s="60"/>
+      <c r="H29" s="60"/>
+      <c r="I29" s="55"/>
       <c r="J29" s="18"/>
       <c r="K29" s="19" t="s">
         <v>117</v>
@@ -6379,13 +6379,13 @@
         <v>50</v>
       </c>
       <c r="B30" s="54"/>
-      <c r="C30" s="61"/>
-      <c r="D30" s="61"/>
-      <c r="E30" s="61"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="61"/>
-      <c r="H30" s="61"/>
-      <c r="I30" s="62"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="60"/>
+      <c r="G30" s="60"/>
+      <c r="H30" s="60"/>
+      <c r="I30" s="55"/>
       <c r="J30" s="18"/>
       <c r="K30" s="19" t="s">
         <v>118</v>
@@ -6396,52 +6396,52 @@
         <v>51</v>
       </c>
       <c r="B31" s="54"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
-      <c r="F31" s="61"/>
-      <c r="G31" s="61"/>
-      <c r="H31" s="61"/>
-      <c r="I31" s="62"/>
+      <c r="C31" s="60"/>
+      <c r="D31" s="60"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="60"/>
+      <c r="G31" s="60"/>
+      <c r="H31" s="60"/>
+      <c r="I31" s="55"/>
       <c r="J31" s="14"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="58"/>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="59"/>
-      <c r="F32" s="59"/>
-      <c r="G32" s="59"/>
-      <c r="H32" s="59"/>
-      <c r="I32" s="60"/>
+      <c r="B32" s="56"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="61"/>
+      <c r="G32" s="61"/>
+      <c r="H32" s="61"/>
+      <c r="I32" s="57"/>
       <c r="J32" s="14"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B33" s="55"/>
-      <c r="C33" s="56"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="56"/>
-      <c r="I33" s="57"/>
+      <c r="B33" s="63"/>
+      <c r="C33" s="58"/>
+      <c r="D33" s="58"/>
+      <c r="E33" s="58"/>
+      <c r="F33" s="58"/>
+      <c r="G33" s="58"/>
+      <c r="H33" s="58"/>
+      <c r="I33" s="59"/>
       <c r="J33" s="14"/>
     </row>
     <row r="34" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="58"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
-      <c r="F34" s="59"/>
-      <c r="G34" s="59"/>
-      <c r="H34" s="59"/>
-      <c r="I34" s="60"/>
+      <c r="B34" s="56"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
+      <c r="I34" s="57"/>
       <c r="J34" s="14"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
@@ -6457,7 +6457,7 @@
       <c r="H35" s="34"/>
       <c r="I35" s="35"/>
       <c r="J35" s="14"/>
-      <c r="K35" s="69" t="s">
+      <c r="K35" s="62" t="s">
         <v>119</v>
       </c>
     </row>
@@ -6474,7 +6474,7 @@
       <c r="H36" s="18"/>
       <c r="I36" s="26"/>
       <c r="J36" s="14"/>
-      <c r="K36" s="69"/>
+      <c r="K36" s="62"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
@@ -6489,7 +6489,7 @@
       <c r="H37" s="18"/>
       <c r="I37" s="26"/>
       <c r="J37" s="14"/>
-      <c r="K37" s="69"/>
+      <c r="K37" s="62"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
@@ -6504,7 +6504,7 @@
       <c r="H38" s="18"/>
       <c r="I38" s="26"/>
       <c r="J38" s="14"/>
-      <c r="K38" s="69" t="s">
+      <c r="K38" s="62" t="s">
         <v>120</v>
       </c>
     </row>
@@ -6521,7 +6521,7 @@
       <c r="H39" s="18"/>
       <c r="I39" s="26"/>
       <c r="J39" s="14"/>
-      <c r="K39" s="69"/>
+      <c r="K39" s="62"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
@@ -6536,7 +6536,7 @@
       <c r="H40" s="18"/>
       <c r="I40" s="26"/>
       <c r="J40" s="14"/>
-      <c r="K40" s="69"/>
+      <c r="K40" s="62"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
@@ -6628,43 +6628,43 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B46" s="54"/>
-      <c r="C46" s="61"/>
-      <c r="D46" s="61"/>
-      <c r="E46" s="61"/>
-      <c r="F46" s="61"/>
-      <c r="G46" s="61"/>
-      <c r="H46" s="61"/>
-      <c r="I46" s="62"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="60"/>
+      <c r="E46" s="60"/>
+      <c r="F46" s="60"/>
+      <c r="G46" s="60"/>
+      <c r="H46" s="60"/>
+      <c r="I46" s="55"/>
       <c r="J46" s="14"/>
     </row>
     <row r="47" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="58"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="59"/>
-      <c r="E47" s="59"/>
-      <c r="F47" s="59"/>
-      <c r="G47" s="59"/>
-      <c r="H47" s="59"/>
-      <c r="I47" s="60"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="61"/>
+      <c r="D47" s="61"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="61"/>
+      <c r="G47" s="61"/>
+      <c r="H47" s="61"/>
+      <c r="I47" s="57"/>
       <c r="J47" s="14"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B48" s="55" t="s">
+      <c r="B48" s="63" t="s">
         <v>179</v>
       </c>
-      <c r="C48" s="56"/>
-      <c r="D48" s="56"/>
-      <c r="E48" s="56"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="56"/>
-      <c r="H48" s="56"/>
-      <c r="I48" s="57"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="58"/>
+      <c r="H48" s="58"/>
+      <c r="I48" s="59"/>
       <c r="J48" s="14"/>
       <c r="K48" s="19" t="s">
         <v>41</v>
@@ -6677,13 +6677,13 @@
       <c r="B49" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C49" s="61"/>
-      <c r="D49" s="61"/>
-      <c r="E49" s="61"/>
-      <c r="F49" s="61"/>
-      <c r="G49" s="61"/>
-      <c r="H49" s="61"/>
-      <c r="I49" s="62"/>
+      <c r="C49" s="60"/>
+      <c r="D49" s="60"/>
+      <c r="E49" s="60"/>
+      <c r="F49" s="60"/>
+      <c r="G49" s="60"/>
+      <c r="H49" s="60"/>
+      <c r="I49" s="55"/>
       <c r="J49" s="14"/>
       <c r="K49" s="19" t="s">
         <v>42</v>
@@ -6696,13 +6696,13 @@
       <c r="B50" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C50" s="61"/>
-      <c r="D50" s="61"/>
-      <c r="E50" s="61"/>
-      <c r="F50" s="61"/>
-      <c r="G50" s="61"/>
-      <c r="H50" s="61"/>
-      <c r="I50" s="62"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="60"/>
+      <c r="E50" s="60"/>
+      <c r="F50" s="60"/>
+      <c r="G50" s="60"/>
+      <c r="H50" s="60"/>
+      <c r="I50" s="55"/>
       <c r="J50" s="14"/>
       <c r="K50" s="19" t="s">
         <v>54</v>
@@ -6715,13 +6715,13 @@
       <c r="B51" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C51" s="61"/>
-      <c r="D51" s="61"/>
-      <c r="E51" s="61"/>
-      <c r="F51" s="61"/>
-      <c r="G51" s="61"/>
-      <c r="H51" s="61"/>
-      <c r="I51" s="62"/>
+      <c r="C51" s="60"/>
+      <c r="D51" s="60"/>
+      <c r="E51" s="60"/>
+      <c r="F51" s="60"/>
+      <c r="G51" s="60"/>
+      <c r="H51" s="60"/>
+      <c r="I51" s="55"/>
       <c r="J51" s="14"/>
       <c r="K51" s="19" t="s">
         <v>74</v>
@@ -6732,19 +6732,19 @@
         <v>158</v>
       </c>
       <c r="B52" s="54"/>
-      <c r="C52" s="61"/>
-      <c r="D52" s="61" t="s">
+      <c r="C52" s="60"/>
+      <c r="D52" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="E52" s="61"/>
-      <c r="F52" s="61" t="s">
+      <c r="E52" s="60"/>
+      <c r="F52" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="G52" s="61"/>
-      <c r="H52" s="61" t="s">
+      <c r="G52" s="60"/>
+      <c r="H52" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="I52" s="62"/>
+      <c r="I52" s="55"/>
       <c r="J52" s="14"/>
       <c r="K52" s="19" t="s">
         <v>124</v>
@@ -6755,19 +6755,19 @@
         <v>157</v>
       </c>
       <c r="B53" s="54"/>
-      <c r="C53" s="61"/>
-      <c r="D53" s="61" t="s">
+      <c r="C53" s="60"/>
+      <c r="D53" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="E53" s="61"/>
-      <c r="F53" s="61" t="s">
+      <c r="E53" s="60"/>
+      <c r="F53" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="G53" s="61"/>
-      <c r="H53" s="61" t="s">
+      <c r="G53" s="60"/>
+      <c r="H53" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="I53" s="62"/>
+      <c r="I53" s="55"/>
       <c r="J53" s="14"/>
       <c r="K53" s="19" t="s">
         <v>159</v>
@@ -6781,15 +6781,15 @@
         <v>84</v>
       </c>
       <c r="C54" s="18"/>
-      <c r="D54" s="61" t="s">
+      <c r="D54" s="60" t="s">
         <v>84</v>
       </c>
       <c r="E54" s="18"/>
-      <c r="F54" s="61" t="s">
+      <c r="F54" s="60" t="s">
         <v>84</v>
       </c>
       <c r="G54" s="18"/>
-      <c r="H54" s="61" t="s">
+      <c r="H54" s="60" t="s">
         <v>84</v>
       </c>
       <c r="I54" s="26"/>
@@ -6804,11 +6804,11 @@
       </c>
       <c r="B55" s="54"/>
       <c r="C55" s="18"/>
-      <c r="D55" s="61"/>
+      <c r="D55" s="60"/>
       <c r="E55" s="18"/>
-      <c r="F55" s="61"/>
+      <c r="F55" s="60"/>
       <c r="G55" s="18"/>
-      <c r="H55" s="61"/>
+      <c r="H55" s="60"/>
       <c r="I55" s="26"/>
       <c r="J55" s="14"/>
       <c r="K55" s="19" t="s">
@@ -6820,23 +6820,23 @@
         <v>155</v>
       </c>
       <c r="B56" s="27"/>
-      <c r="C56" s="61" t="s">
+      <c r="C56" s="60" t="s">
         <v>84</v>
       </c>
       <c r="D56" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="E56" s="61" t="s">
+      <c r="E56" s="60" t="s">
         <v>84</v>
       </c>
       <c r="F56" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="G56" s="61" t="s">
+      <c r="G56" s="60" t="s">
         <v>84</v>
       </c>
       <c r="H56" s="18"/>
-      <c r="I56" s="62" t="s">
+      <c r="I56" s="55" t="s">
         <v>84</v>
       </c>
       <c r="J56" s="14"/>
@@ -6849,55 +6849,55 @@
         <v>162</v>
       </c>
       <c r="B57" s="27"/>
-      <c r="C57" s="59"/>
+      <c r="C57" s="61"/>
       <c r="D57" s="18"/>
-      <c r="E57" s="59"/>
+      <c r="E57" s="61"/>
       <c r="F57" s="18"/>
-      <c r="G57" s="59"/>
+      <c r="G57" s="61"/>
       <c r="H57" s="18"/>
-      <c r="I57" s="60"/>
+      <c r="I57" s="57"/>
       <c r="J57" s="14"/>
       <c r="K57" s="19" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B58" s="55"/>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
-      <c r="I58" s="57"/>
+      <c r="B58" s="63"/>
+      <c r="C58" s="58"/>
+      <c r="D58" s="58"/>
+      <c r="E58" s="58"/>
+      <c r="F58" s="58"/>
+      <c r="G58" s="58"/>
+      <c r="H58" s="58"/>
+      <c r="I58" s="59"/>
       <c r="J58" s="14"/>
     </row>
     <row r="59" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B59" s="58"/>
-      <c r="C59" s="59"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="59"/>
-      <c r="F59" s="59"/>
-      <c r="G59" s="59"/>
-      <c r="H59" s="59"/>
-      <c r="I59" s="60"/>
+      <c r="B59" s="56"/>
+      <c r="C59" s="61"/>
+      <c r="D59" s="61"/>
+      <c r="E59" s="61"/>
+      <c r="F59" s="61"/>
+      <c r="G59" s="61"/>
+      <c r="H59" s="61"/>
+      <c r="I59" s="57"/>
       <c r="J59" s="14"/>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="55"/>
-      <c r="C60" s="56"/>
-      <c r="D60" s="56"/>
-      <c r="E60" s="56"/>
-      <c r="F60" s="56"/>
-      <c r="G60" s="56"/>
-      <c r="H60" s="56"/>
-      <c r="I60" s="57"/>
+      <c r="B60" s="63"/>
+      <c r="C60" s="58"/>
+      <c r="D60" s="58"/>
+      <c r="E60" s="58"/>
+      <c r="F60" s="58"/>
+      <c r="G60" s="58"/>
+      <c r="H60" s="58"/>
+      <c r="I60" s="59"/>
       <c r="J60" s="14"/>
       <c r="K60" s="19" t="s">
         <v>127</v>
@@ -6909,13 +6909,13 @@
         <v>45</v>
       </c>
       <c r="B61" s="54"/>
-      <c r="C61" s="61"/>
-      <c r="D61" s="61"/>
-      <c r="E61" s="61"/>
-      <c r="F61" s="61"/>
-      <c r="G61" s="61"/>
-      <c r="H61" s="61"/>
-      <c r="I61" s="62"/>
+      <c r="C61" s="60"/>
+      <c r="D61" s="60"/>
+      <c r="E61" s="60"/>
+      <c r="F61" s="60"/>
+      <c r="G61" s="60"/>
+      <c r="H61" s="60"/>
+      <c r="I61" s="55"/>
       <c r="J61" s="14"/>
       <c r="K61" s="19" t="s">
         <v>128</v>
@@ -6926,17 +6926,17 @@
         <v>86</v>
       </c>
       <c r="B62" s="54"/>
-      <c r="C62" s="61"/>
-      <c r="D62" s="61" t="s">
+      <c r="C62" s="60"/>
+      <c r="D62" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="E62" s="61"/>
-      <c r="F62" s="61"/>
-      <c r="G62" s="61"/>
-      <c r="H62" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="I62" s="62"/>
+      <c r="E62" s="60"/>
+      <c r="F62" s="60"/>
+      <c r="G62" s="60"/>
+      <c r="H62" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="I62" s="55"/>
       <c r="J62" s="14"/>
       <c r="K62" s="19" t="s">
         <v>129</v>
@@ -6947,15 +6947,15 @@
         <v>152</v>
       </c>
       <c r="B63" s="54"/>
-      <c r="C63" s="61"/>
-      <c r="D63" s="61" t="s">
+      <c r="C63" s="60"/>
+      <c r="D63" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="E63" s="61"/>
-      <c r="F63" s="61"/>
-      <c r="G63" s="61"/>
-      <c r="H63" s="61"/>
-      <c r="I63" s="62"/>
+      <c r="E63" s="60"/>
+      <c r="F63" s="60"/>
+      <c r="G63" s="60"/>
+      <c r="H63" s="60"/>
+      <c r="I63" s="55"/>
       <c r="J63" s="14"/>
       <c r="K63" s="19" t="s">
         <v>130</v>
@@ -6971,10 +6971,10 @@
       <c r="E64" s="18"/>
       <c r="F64" s="18"/>
       <c r="G64" s="18"/>
-      <c r="H64" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="I64" s="62"/>
+      <c r="H64" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="I64" s="55"/>
       <c r="J64" s="14"/>
       <c r="K64" s="19" t="s">
         <v>131</v>
@@ -6985,13 +6985,13 @@
         <v>93</v>
       </c>
       <c r="B65" s="54"/>
-      <c r="C65" s="61"/>
-      <c r="D65" s="61"/>
-      <c r="E65" s="61"/>
-      <c r="F65" s="61"/>
-      <c r="G65" s="61"/>
-      <c r="H65" s="61"/>
-      <c r="I65" s="62"/>
+      <c r="C65" s="60"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="60"/>
+      <c r="F65" s="60"/>
+      <c r="G65" s="60"/>
+      <c r="H65" s="60"/>
+      <c r="I65" s="55"/>
       <c r="J65" s="14"/>
       <c r="K65" s="19" t="s">
         <v>132</v>
@@ -7001,20 +7001,20 @@
       <c r="A66" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B66" s="55"/>
-      <c r="C66" s="56"/>
-      <c r="D66" s="56" t="s">
+      <c r="B66" s="63"/>
+      <c r="C66" s="58"/>
+      <c r="D66" s="58" t="s">
         <v>83</v>
       </c>
-      <c r="E66" s="56"/>
-      <c r="F66" s="56"/>
-      <c r="G66" s="56"/>
-      <c r="H66" s="56" t="s">
-        <v>84</v>
-      </c>
-      <c r="I66" s="57"/>
+      <c r="E66" s="58"/>
+      <c r="F66" s="58"/>
+      <c r="G66" s="58"/>
+      <c r="H66" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="I66" s="59"/>
       <c r="J66" s="14"/>
-      <c r="K66" s="69" t="s">
+      <c r="K66" s="62" t="s">
         <v>133</v>
       </c>
     </row>
@@ -7023,28 +7023,28 @@
         <v>139</v>
       </c>
       <c r="B67" s="54"/>
-      <c r="C67" s="61"/>
-      <c r="D67" s="61"/>
-      <c r="E67" s="61"/>
-      <c r="F67" s="61"/>
-      <c r="G67" s="61"/>
-      <c r="H67" s="61"/>
-      <c r="I67" s="62"/>
+      <c r="C67" s="60"/>
+      <c r="D67" s="60"/>
+      <c r="E67" s="60"/>
+      <c r="F67" s="60"/>
+      <c r="G67" s="60"/>
+      <c r="H67" s="60"/>
+      <c r="I67" s="55"/>
       <c r="J67" s="14"/>
-      <c r="K67" s="69"/>
+      <c r="K67" s="62"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" s="7" t="s">
         <v>143</v>
       </c>
       <c r="B68" s="54"/>
-      <c r="C68" s="61"/>
-      <c r="D68" s="61"/>
-      <c r="E68" s="61"/>
-      <c r="F68" s="61"/>
-      <c r="G68" s="61"/>
-      <c r="H68" s="61"/>
-      <c r="I68" s="62"/>
+      <c r="C68" s="60"/>
+      <c r="D68" s="60"/>
+      <c r="E68" s="60"/>
+      <c r="F68" s="60"/>
+      <c r="G68" s="60"/>
+      <c r="H68" s="60"/>
+      <c r="I68" s="55"/>
       <c r="J68" s="14"/>
       <c r="K68" s="19" t="s">
         <v>134</v>
@@ -7055,13 +7055,13 @@
         <v>142</v>
       </c>
       <c r="B69" s="54"/>
-      <c r="C69" s="61"/>
-      <c r="D69" s="61"/>
-      <c r="E69" s="61"/>
-      <c r="F69" s="61"/>
-      <c r="G69" s="61"/>
-      <c r="H69" s="61"/>
-      <c r="I69" s="62"/>
+      <c r="C69" s="60"/>
+      <c r="D69" s="60"/>
+      <c r="E69" s="60"/>
+      <c r="F69" s="60"/>
+      <c r="G69" s="60"/>
+      <c r="H69" s="60"/>
+      <c r="I69" s="55"/>
       <c r="J69" s="14"/>
       <c r="K69" s="19" t="s">
         <v>135</v>
@@ -7071,14 +7071,14 @@
       <c r="A70" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B70" s="58"/>
-      <c r="C70" s="59"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="59"/>
-      <c r="F70" s="59"/>
-      <c r="G70" s="59"/>
-      <c r="H70" s="59"/>
-      <c r="I70" s="60"/>
+      <c r="B70" s="56"/>
+      <c r="C70" s="61"/>
+      <c r="D70" s="61"/>
+      <c r="E70" s="61"/>
+      <c r="F70" s="61"/>
+      <c r="G70" s="61"/>
+      <c r="H70" s="61"/>
+      <c r="I70" s="57"/>
       <c r="J70" s="14"/>
       <c r="K70" s="19" t="s">
         <v>133</v>
@@ -7091,19 +7091,19 @@
       <c r="B71" s="54" t="s">
         <v>179</v>
       </c>
-      <c r="C71" s="61"/>
-      <c r="D71" s="61" t="s">
+      <c r="C71" s="60"/>
+      <c r="D71" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="E71" s="61"/>
-      <c r="F71" s="61" t="s">
+      <c r="E71" s="60"/>
+      <c r="F71" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="G71" s="61"/>
-      <c r="H71" s="56" t="s">
-        <v>84</v>
-      </c>
-      <c r="I71" s="57"/>
+      <c r="G71" s="60"/>
+      <c r="H71" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="I71" s="59"/>
       <c r="J71" s="14"/>
       <c r="K71" s="19" t="s">
         <v>137</v>
@@ -7113,20 +7113,20 @@
       <c r="A72" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B72" s="63" t="s">
+      <c r="B72" s="67" t="s">
         <v>179</v>
       </c>
-      <c r="C72" s="64"/>
-      <c r="D72" s="64" t="s">
+      <c r="C72" s="68"/>
+      <c r="D72" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="E72" s="64"/>
-      <c r="F72" s="64" t="s">
+      <c r="E72" s="68"/>
+      <c r="F72" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="G72" s="64"/>
-      <c r="H72" s="64"/>
-      <c r="I72" s="65"/>
+      <c r="G72" s="68"/>
+      <c r="H72" s="68"/>
+      <c r="I72" s="69"/>
       <c r="J72" s="14"/>
       <c r="K72" s="19" t="s">
         <v>136</v>
@@ -7134,6 +7134,99 @@
     </row>
   </sheetData>
   <mergeCells count="113">
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="B25:I26"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="B33:I34"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="K35:K37"/>
+    <mergeCell ref="K38:K40"/>
+    <mergeCell ref="B46:I47"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="F54:F55"/>
+    <mergeCell ref="H54:H55"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="I56:I57"/>
+    <mergeCell ref="B58:I59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="K66:K67"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="H65:I65"/>
+    <mergeCell ref="H64:I64"/>
+    <mergeCell ref="H62:I63"/>
     <mergeCell ref="B72:C72"/>
     <mergeCell ref="D72:E72"/>
     <mergeCell ref="F72:G72"/>
@@ -7154,99 +7247,6 @@
     <mergeCell ref="F69:G69"/>
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="D66:E66"/>
-    <mergeCell ref="K66:K67"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="D63:E63"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="H65:I65"/>
-    <mergeCell ref="H64:I64"/>
-    <mergeCell ref="H62:I63"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="H61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="G56:G57"/>
-    <mergeCell ref="I56:I57"/>
-    <mergeCell ref="B58:I59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="F54:F55"/>
-    <mergeCell ref="H54:H55"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="K35:K37"/>
-    <mergeCell ref="K38:K40"/>
-    <mergeCell ref="B46:I47"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="B33:I34"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="B25:I26"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:I59 B60:D60 F60 H60 B61:I61 B62:H62 B63:G63 B64:H64 B65:I65 B66:F66 H66 B67:G70 B71:H71 B72:G72">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">

</xml_diff>